<commit_message>
feat: Normalización a escala 100 de los índices en los 3 grupos poblacionales
</commit_message>
<xml_diff>
--- a/output/df_docentes_final.xlsx
+++ b/output/df_docentes_final.xlsx
@@ -459,12 +459,12 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Indice_Conocimiento</t>
+          <t>Indice_Conocimiento_Norm</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Indice_Capacidades_Respuesta</t>
+          <t>Indice_Capacidades_Respuesta_Norm</t>
         </is>
       </c>
     </row>
@@ -510,10 +510,10 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>46</v>
+        <v>83.63636363636363</v>
       </c>
       <c r="J2" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
@@ -558,10 +558,10 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>30</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="J3" t="n">
-        <v>23</v>
+        <v>76.66666666666667</v>
       </c>
     </row>
     <row r="4">
@@ -606,10 +606,10 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>27</v>
+        <v>49.09090909090909</v>
       </c>
       <c r="J4" t="n">
-        <v>5</v>
+        <v>16.66666666666666</v>
       </c>
     </row>
     <row r="5">
@@ -654,10 +654,10 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>49</v>
+        <v>89.09090909090909</v>
       </c>
       <c r="J5" t="n">
-        <v>29</v>
+        <v>96.66666666666667</v>
       </c>
     </row>
     <row r="6">
@@ -702,10 +702,10 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>28</v>
+        <v>50.90909090909091</v>
       </c>
       <c r="J6" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
@@ -750,10 +750,10 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>27</v>
+        <v>49.09090909090909</v>
       </c>
       <c r="J7" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="8">
@@ -798,10 +798,10 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>28</v>
+        <v>50.90909090909091</v>
       </c>
       <c r="J8" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9">
@@ -846,10 +846,10 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>29</v>
+        <v>52.72727272727272</v>
       </c>
       <c r="J9" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="10">
@@ -894,10 +894,10 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>35</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="J10" t="n">
-        <v>11</v>
+        <v>36.66666666666666</v>
       </c>
     </row>
     <row r="11">
@@ -942,10 +942,10 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>32</v>
+        <v>58.18181818181818</v>
       </c>
       <c r="J11" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12">
@@ -990,10 +990,10 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="J12" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13">
@@ -1038,10 +1038,10 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>26</v>
+        <v>47.27272727272727</v>
       </c>
       <c r="J13" t="n">
-        <v>20</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="14">
@@ -1086,10 +1086,10 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J14" t="n">
-        <v>16</v>
+        <v>53.33333333333334</v>
       </c>
     </row>
     <row r="15">
@@ -1134,10 +1134,10 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>34</v>
+        <v>61.81818181818181</v>
       </c>
       <c r="J15" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16">
@@ -1182,10 +1182,10 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>36</v>
+        <v>65.45454545454545</v>
       </c>
       <c r="J16" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17">
@@ -1230,10 +1230,10 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>30</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="J17" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="18">
@@ -1278,10 +1278,10 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>24</v>
+        <v>43.63636363636363</v>
       </c>
       <c r="J18" t="n">
-        <v>20</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="19">
@@ -1326,10 +1326,10 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>37</v>
+        <v>67.27272727272727</v>
       </c>
       <c r="J19" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="20">
@@ -1374,10 +1374,10 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>30</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="J20" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21">
@@ -1422,10 +1422,10 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>39</v>
+        <v>70.90909090909091</v>
       </c>
       <c r="J21" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="22">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>19</v>
+        <v>34.54545454545455</v>
       </c>
       <c r="J22" t="n">
-        <v>11</v>
+        <v>36.66666666666666</v>
       </c>
     </row>
     <row r="23">
@@ -1518,10 +1518,10 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>81.81818181818183</v>
       </c>
       <c r="J23" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>27</v>
+        <v>49.09090909090909</v>
       </c>
       <c r="J24" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="25">
@@ -1614,10 +1614,10 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>35</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="J25" t="n">
-        <v>11</v>
+        <v>36.66666666666666</v>
       </c>
     </row>
     <row r="26">
@@ -1662,10 +1662,10 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>32</v>
+        <v>58.18181818181818</v>
       </c>
       <c r="J26" t="n">
-        <v>20</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="27">
@@ -1710,10 +1710,10 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>40</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="J27" t="n">
-        <v>26</v>
+        <v>86.66666666666667</v>
       </c>
     </row>
     <row r="28">
@@ -1758,10 +1758,10 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="J28" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="29">
@@ -1806,10 +1806,10 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>32</v>
+        <v>58.18181818181818</v>
       </c>
       <c r="J29" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30">
@@ -1854,10 +1854,10 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>27</v>
+        <v>49.09090909090909</v>
       </c>
       <c r="J30" t="n">
-        <v>14</v>
+        <v>46.66666666666666</v>
       </c>
     </row>
     <row r="31">
@@ -1902,10 +1902,10 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>36</v>
+        <v>65.45454545454545</v>
       </c>
       <c r="J31" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32">
@@ -1950,10 +1950,10 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>39</v>
+        <v>70.90909090909091</v>
       </c>
       <c r="J32" t="n">
-        <v>14</v>
+        <v>46.66666666666666</v>
       </c>
     </row>
     <row r="33">
@@ -1998,10 +1998,10 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>36</v>
+        <v>65.45454545454545</v>
       </c>
       <c r="J33" t="n">
-        <v>8</v>
+        <v>26.66666666666667</v>
       </c>
     </row>
     <row r="34">
@@ -2046,10 +2046,10 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>39</v>
+        <v>70.90909090909091</v>
       </c>
       <c r="J34" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="35">
@@ -2094,10 +2094,10 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>35</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="J35" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="36">
@@ -2142,10 +2142,10 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="J36" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37">
@@ -2190,10 +2190,10 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>32</v>
+        <v>58.18181818181818</v>
       </c>
       <c r="J37" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="38">
@@ -2238,10 +2238,10 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>24</v>
+        <v>43.63636363636363</v>
       </c>
       <c r="J38" t="n">
-        <v>23</v>
+        <v>76.66666666666667</v>
       </c>
     </row>
     <row r="39">
@@ -2286,10 +2286,10 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>29</v>
+        <v>52.72727272727272</v>
       </c>
       <c r="J39" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="40">
@@ -2334,10 +2334,10 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>41</v>
+        <v>74.54545454545455</v>
       </c>
       <c r="J40" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="41">
@@ -2382,10 +2382,10 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>38</v>
+        <v>69.09090909090909</v>
       </c>
       <c r="J41" t="n">
-        <v>20</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="42">
@@ -2430,10 +2430,10 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>49</v>
+        <v>89.09090909090909</v>
       </c>
       <c r="J42" t="n">
-        <v>26</v>
+        <v>86.66666666666667</v>
       </c>
     </row>
     <row r="43">
@@ -2478,10 +2478,10 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>41</v>
+        <v>74.54545454545455</v>
       </c>
       <c r="J43" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="44">
@@ -2526,10 +2526,10 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="J44" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="45">
@@ -2574,10 +2574,10 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>42</v>
+        <v>76.36363636363637</v>
       </c>
       <c r="J45" t="n">
-        <v>13</v>
+        <v>43.33333333333334</v>
       </c>
     </row>
     <row r="46">
@@ -2622,10 +2622,10 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>30</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="J46" t="n">
-        <v>8</v>
+        <v>26.66666666666667</v>
       </c>
     </row>
     <row r="47">
@@ -2670,10 +2670,10 @@
         </is>
       </c>
       <c r="I47" t="n">
-        <v>37</v>
+        <v>67.27272727272727</v>
       </c>
       <c r="J47" t="n">
-        <v>20</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="48">
@@ -2718,10 +2718,10 @@
         </is>
       </c>
       <c r="I48" t="n">
-        <v>53</v>
+        <v>96.36363636363636</v>
       </c>
       <c r="J48" t="n">
-        <v>20</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="49">
@@ -2766,10 +2766,10 @@
         </is>
       </c>
       <c r="I49" t="n">
-        <v>38</v>
+        <v>69.09090909090909</v>
       </c>
       <c r="J49" t="n">
-        <v>20</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="50">
@@ -2814,10 +2814,10 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J50" t="n">
-        <v>17</v>
+        <v>56.66666666666666</v>
       </c>
     </row>
     <row r="51">
@@ -2862,10 +2862,10 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>25</v>
+        <v>45.45454545454545</v>
       </c>
       <c r="J51" t="n">
-        <v>25</v>
+        <v>83.33333333333334</v>
       </c>
     </row>
     <row r="52">
@@ -2910,10 +2910,10 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>37</v>
+        <v>67.27272727272727</v>
       </c>
       <c r="J52" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="53">
@@ -2958,10 +2958,10 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J53" t="n">
-        <v>20</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="54">
@@ -3006,10 +3006,10 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>42</v>
+        <v>76.36363636363637</v>
       </c>
       <c r="J54" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="55">
@@ -3054,10 +3054,10 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>37</v>
+        <v>67.27272727272727</v>
       </c>
       <c r="J55" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="56">
@@ -3102,10 +3102,10 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>32</v>
+        <v>58.18181818181818</v>
       </c>
       <c r="J56" t="n">
-        <v>14</v>
+        <v>46.66666666666666</v>
       </c>
     </row>
     <row r="57">
@@ -3150,7 +3150,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>14</v>
+        <v>25.45454545454545</v>
       </c>
       <c r="J57" t="n">
         <v>0</v>
@@ -3198,10 +3198,10 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>49</v>
+        <v>89.09090909090909</v>
       </c>
       <c r="J58" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="59">
@@ -3246,10 +3246,10 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>27</v>
+        <v>49.09090909090909</v>
       </c>
       <c r="J59" t="n">
-        <v>13</v>
+        <v>43.33333333333334</v>
       </c>
     </row>
     <row r="60">
@@ -3294,10 +3294,10 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>46</v>
+        <v>83.63636363636363</v>
       </c>
       <c r="J60" t="n">
-        <v>23</v>
+        <v>76.66666666666667</v>
       </c>
     </row>
     <row r="61">
@@ -3342,10 +3342,10 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="J61" t="n">
-        <v>13</v>
+        <v>43.33333333333334</v>
       </c>
     </row>
     <row r="62">
@@ -3390,10 +3390,10 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>37</v>
+        <v>67.27272727272727</v>
       </c>
       <c r="J62" t="n">
-        <v>28</v>
+        <v>93.33333333333333</v>
       </c>
     </row>
     <row r="63">
@@ -3438,10 +3438,10 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>37</v>
+        <v>67.27272727272727</v>
       </c>
       <c r="J63" t="n">
-        <v>13</v>
+        <v>43.33333333333334</v>
       </c>
     </row>
     <row r="64">
@@ -3486,10 +3486,10 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>42</v>
+        <v>76.36363636363637</v>
       </c>
       <c r="J64" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="65">
@@ -3534,10 +3534,10 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="J65" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
     </row>
     <row r="66">
@@ -3582,10 +3582,10 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>30</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="J66" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
     </row>
     <row r="67">
@@ -3630,10 +3630,10 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="J67" t="n">
-        <v>1</v>
+        <v>3.333333333333333</v>
       </c>
     </row>
     <row r="68">
@@ -3678,10 +3678,10 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>29</v>
+        <v>52.72727272727272</v>
       </c>
       <c r="J68" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="69">
@@ -3726,10 +3726,10 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J69" t="n">
-        <v>14</v>
+        <v>46.66666666666666</v>
       </c>
     </row>
     <row r="70">
@@ -3774,10 +3774,10 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>30</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="J70" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="71">
@@ -3822,10 +3822,10 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="J71" t="n">
-        <v>25</v>
+        <v>83.33333333333334</v>
       </c>
     </row>
     <row r="72">
@@ -3870,10 +3870,10 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>39</v>
+        <v>70.90909090909091</v>
       </c>
       <c r="J72" t="n">
-        <v>26</v>
+        <v>86.66666666666667</v>
       </c>
     </row>
     <row r="73">
@@ -3918,10 +3918,10 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>25</v>
+        <v>45.45454545454545</v>
       </c>
       <c r="J73" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="74">
@@ -3966,10 +3966,10 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>25</v>
+        <v>45.45454545454545</v>
       </c>
       <c r="J74" t="n">
-        <v>11</v>
+        <v>36.66666666666666</v>
       </c>
     </row>
     <row r="75">
@@ -4014,10 +4014,10 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>41</v>
+        <v>74.54545454545455</v>
       </c>
       <c r="J75" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
     </row>
     <row r="76">
@@ -4062,10 +4062,10 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>32</v>
+        <v>58.18181818181818</v>
       </c>
       <c r="J76" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="77">
@@ -4110,10 +4110,10 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="J77" t="n">
-        <v>25</v>
+        <v>83.33333333333334</v>
       </c>
     </row>
     <row r="78">
@@ -4158,10 +4158,10 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>28</v>
+        <v>50.90909090909091</v>
       </c>
       <c r="J78" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="79">
@@ -4206,10 +4206,10 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J79" t="n">
-        <v>16</v>
+        <v>53.33333333333334</v>
       </c>
     </row>
     <row r="80">
@@ -4254,10 +4254,10 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>30</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="J80" t="n">
-        <v>16</v>
+        <v>53.33333333333334</v>
       </c>
     </row>
     <row r="81">
@@ -4302,10 +4302,10 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J81" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="82">
@@ -4350,10 +4350,10 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>36</v>
+        <v>65.45454545454545</v>
       </c>
       <c r="J82" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="83">
@@ -4398,10 +4398,10 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>38</v>
+        <v>69.09090909090909</v>
       </c>
       <c r="J83" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="84">
@@ -4446,10 +4446,10 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J84" t="n">
-        <v>10</v>
+        <v>33.33333333333333</v>
       </c>
     </row>
     <row r="85">
@@ -4494,10 +4494,10 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>40</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="J85" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="86">
@@ -4542,10 +4542,10 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>36</v>
+        <v>65.45454545454545</v>
       </c>
       <c r="J86" t="n">
-        <v>23</v>
+        <v>76.66666666666667</v>
       </c>
     </row>
     <row r="87">
@@ -4590,10 +4590,10 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J87" t="n">
-        <v>7</v>
+        <v>23.33333333333333</v>
       </c>
     </row>
     <row r="88">
@@ -4638,10 +4638,10 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>39</v>
+        <v>70.90909090909091</v>
       </c>
       <c r="J88" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="89">
@@ -4686,7 +4686,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>13</v>
+        <v>23.63636363636364</v>
       </c>
       <c r="J89" t="n">
         <v>0</v>
@@ -4734,10 +4734,10 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>32</v>
+        <v>58.18181818181818</v>
       </c>
       <c r="J90" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="91">
@@ -4782,10 +4782,10 @@
         </is>
       </c>
       <c r="I91" t="n">
-        <v>39</v>
+        <v>70.90909090909091</v>
       </c>
       <c r="J91" t="n">
-        <v>26</v>
+        <v>86.66666666666667</v>
       </c>
     </row>
     <row r="92">
@@ -4830,10 +4830,10 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>35</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="J92" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="93">
@@ -4878,10 +4878,10 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>26</v>
+        <v>47.27272727272727</v>
       </c>
       <c r="J93" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="94">
@@ -4926,10 +4926,10 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>29</v>
+        <v>52.72727272727272</v>
       </c>
       <c r="J94" t="n">
-        <v>13</v>
+        <v>43.33333333333334</v>
       </c>
     </row>
     <row r="95">
@@ -4974,10 +4974,10 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>32</v>
+        <v>58.18181818181818</v>
       </c>
       <c r="J95" t="n">
-        <v>13</v>
+        <v>43.33333333333334</v>
       </c>
     </row>
     <row r="96">
@@ -5022,10 +5022,10 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>41</v>
+        <v>74.54545454545455</v>
       </c>
       <c r="J96" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="97">
@@ -5070,10 +5070,10 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="J97" t="n">
-        <v>10</v>
+        <v>33.33333333333333</v>
       </c>
     </row>
     <row r="98">
@@ -5118,10 +5118,10 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>38</v>
+        <v>69.09090909090909</v>
       </c>
       <c r="J98" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="99">
@@ -5166,10 +5166,10 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="J99" t="n">
-        <v>24</v>
+        <v>80</v>
       </c>
     </row>
     <row r="100">
@@ -5214,10 +5214,10 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>27</v>
+        <v>49.09090909090909</v>
       </c>
       <c r="J100" t="n">
-        <v>14</v>
+        <v>46.66666666666666</v>
       </c>
     </row>
     <row r="101">
@@ -5262,10 +5262,10 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>32</v>
+        <v>58.18181818181818</v>
       </c>
       <c r="J101" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
     </row>
     <row r="102">
@@ -5310,10 +5310,10 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>29</v>
+        <v>52.72727272727272</v>
       </c>
       <c r="J102" t="n">
-        <v>20</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="103">
@@ -5358,10 +5358,10 @@
         </is>
       </c>
       <c r="I103" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J103" t="n">
-        <v>27</v>
+        <v>90</v>
       </c>
     </row>
     <row r="104">
@@ -5406,10 +5406,10 @@
         </is>
       </c>
       <c r="I104" t="n">
-        <v>25</v>
+        <v>45.45454545454545</v>
       </c>
       <c r="J104" t="n">
-        <v>10</v>
+        <v>33.33333333333333</v>
       </c>
     </row>
     <row r="105">
@@ -5454,10 +5454,10 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>32</v>
+        <v>58.18181818181818</v>
       </c>
       <c r="J105" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
     </row>
     <row r="106">
@@ -5502,10 +5502,10 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>36</v>
+        <v>65.45454545454545</v>
       </c>
       <c r="J106" t="n">
-        <v>17</v>
+        <v>56.66666666666666</v>
       </c>
     </row>
     <row r="107">
@@ -5550,10 +5550,10 @@
         </is>
       </c>
       <c r="I107" t="n">
-        <v>46</v>
+        <v>83.63636363636363</v>
       </c>
       <c r="J107" t="n">
-        <v>28</v>
+        <v>93.33333333333333</v>
       </c>
     </row>
     <row r="108">
@@ -5598,10 +5598,10 @@
         </is>
       </c>
       <c r="I108" t="n">
-        <v>27</v>
+        <v>49.09090909090909</v>
       </c>
       <c r="J108" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="109">
@@ -5646,10 +5646,10 @@
         </is>
       </c>
       <c r="I109" t="n">
-        <v>24</v>
+        <v>43.63636363636363</v>
       </c>
       <c r="J109" t="n">
-        <v>10</v>
+        <v>33.33333333333333</v>
       </c>
     </row>
     <row r="110">
@@ -5694,10 +5694,10 @@
         </is>
       </c>
       <c r="I110" t="n">
-        <v>38</v>
+        <v>69.09090909090909</v>
       </c>
       <c r="J110" t="n">
-        <v>24</v>
+        <v>80</v>
       </c>
     </row>
     <row r="111">
@@ -5742,10 +5742,10 @@
         </is>
       </c>
       <c r="I111" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="J111" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="112">
@@ -5790,10 +5790,10 @@
         </is>
       </c>
       <c r="I112" t="n">
-        <v>40</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="J112" t="n">
-        <v>27</v>
+        <v>90</v>
       </c>
     </row>
     <row r="113">
@@ -5838,10 +5838,10 @@
         </is>
       </c>
       <c r="I113" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J113" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="114">
@@ -5886,10 +5886,10 @@
         </is>
       </c>
       <c r="I114" t="n">
-        <v>40</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="J114" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="115">
@@ -5934,10 +5934,10 @@
         </is>
       </c>
       <c r="I115" t="n">
-        <v>45</v>
+        <v>81.81818181818183</v>
       </c>
       <c r="J115" t="n">
-        <v>23</v>
+        <v>76.66666666666667</v>
       </c>
     </row>
     <row r="116">
@@ -5982,10 +5982,10 @@
         </is>
       </c>
       <c r="I116" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J116" t="n">
-        <v>25</v>
+        <v>83.33333333333334</v>
       </c>
     </row>
     <row r="117">
@@ -6030,10 +6030,10 @@
         </is>
       </c>
       <c r="I117" t="n">
-        <v>38</v>
+        <v>69.09090909090909</v>
       </c>
       <c r="J117" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="118">
@@ -6078,10 +6078,10 @@
         </is>
       </c>
       <c r="I118" t="n">
-        <v>39</v>
+        <v>70.90909090909091</v>
       </c>
       <c r="J118" t="n">
-        <v>26</v>
+        <v>86.66666666666667</v>
       </c>
     </row>
     <row r="119">
@@ -6126,10 +6126,10 @@
         </is>
       </c>
       <c r="I119" t="n">
-        <v>26</v>
+        <v>47.27272727272727</v>
       </c>
       <c r="J119" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="120">
@@ -6174,10 +6174,10 @@
         </is>
       </c>
       <c r="I120" t="n">
-        <v>37</v>
+        <v>67.27272727272727</v>
       </c>
       <c r="J120" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="121">
@@ -6222,10 +6222,10 @@
         </is>
       </c>
       <c r="I121" t="n">
-        <v>23</v>
+        <v>41.81818181818181</v>
       </c>
       <c r="J121" t="n">
-        <v>13</v>
+        <v>43.33333333333334</v>
       </c>
     </row>
     <row r="122">
@@ -6270,10 +6270,10 @@
         </is>
       </c>
       <c r="I122" t="n">
-        <v>32</v>
+        <v>58.18181818181818</v>
       </c>
       <c r="J122" t="n">
-        <v>16</v>
+        <v>53.33333333333334</v>
       </c>
     </row>
     <row r="123">
@@ -6318,10 +6318,10 @@
         </is>
       </c>
       <c r="I123" t="n">
-        <v>27</v>
+        <v>49.09090909090909</v>
       </c>
       <c r="J123" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="124">
@@ -6366,10 +6366,10 @@
         </is>
       </c>
       <c r="I124" t="n">
-        <v>32</v>
+        <v>58.18181818181818</v>
       </c>
       <c r="J124" t="n">
-        <v>25</v>
+        <v>83.33333333333334</v>
       </c>
     </row>
     <row r="125">
@@ -6414,10 +6414,10 @@
         </is>
       </c>
       <c r="I125" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="J125" t="n">
-        <v>24</v>
+        <v>80</v>
       </c>
     </row>
     <row r="126">
@@ -6462,10 +6462,10 @@
         </is>
       </c>
       <c r="I126" t="n">
-        <v>28</v>
+        <v>50.90909090909091</v>
       </c>
       <c r="J126" t="n">
-        <v>20</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="127">
@@ -6510,10 +6510,10 @@
         </is>
       </c>
       <c r="I127" t="n">
-        <v>51</v>
+        <v>92.72727272727272</v>
       </c>
       <c r="J127" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
     </row>
     <row r="128">
@@ -6558,10 +6558,10 @@
         </is>
       </c>
       <c r="I128" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="J128" t="n">
-        <v>11</v>
+        <v>36.66666666666666</v>
       </c>
     </row>
     <row r="129">
@@ -6606,10 +6606,10 @@
         </is>
       </c>
       <c r="I129" t="n">
-        <v>30</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="J129" t="n">
-        <v>13</v>
+        <v>43.33333333333334</v>
       </c>
     </row>
     <row r="130">
@@ -6654,10 +6654,10 @@
         </is>
       </c>
       <c r="I130" t="n">
-        <v>34</v>
+        <v>61.81818181818181</v>
       </c>
       <c r="J130" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="131">
@@ -6702,10 +6702,10 @@
         </is>
       </c>
       <c r="I131" t="n">
-        <v>45</v>
+        <v>81.81818181818183</v>
       </c>
       <c r="J131" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="132">
@@ -6750,10 +6750,10 @@
         </is>
       </c>
       <c r="I132" t="n">
-        <v>21</v>
+        <v>38.18181818181819</v>
       </c>
       <c r="J132" t="n">
-        <v>8</v>
+        <v>26.66666666666667</v>
       </c>
     </row>
     <row r="133">
@@ -6798,10 +6798,10 @@
         </is>
       </c>
       <c r="I133" t="n">
-        <v>40</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="J133" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="134">
@@ -6846,10 +6846,10 @@
         </is>
       </c>
       <c r="I134" t="n">
-        <v>51</v>
+        <v>92.72727272727272</v>
       </c>
       <c r="J134" t="n">
-        <v>25</v>
+        <v>83.33333333333334</v>
       </c>
     </row>
     <row r="135">
@@ -6894,10 +6894,10 @@
         </is>
       </c>
       <c r="I135" t="n">
-        <v>28</v>
+        <v>50.90909090909091</v>
       </c>
       <c r="J135" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="136">
@@ -6942,10 +6942,10 @@
         </is>
       </c>
       <c r="I136" t="n">
-        <v>34</v>
+        <v>61.81818181818181</v>
       </c>
       <c r="J136" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="137">
@@ -6990,10 +6990,10 @@
         </is>
       </c>
       <c r="I137" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J137" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="138">
@@ -7038,10 +7038,10 @@
         </is>
       </c>
       <c r="I138" t="n">
-        <v>28</v>
+        <v>50.90909090909091</v>
       </c>
       <c r="J138" t="n">
-        <v>10</v>
+        <v>33.33333333333333</v>
       </c>
     </row>
     <row r="139">
@@ -7086,10 +7086,10 @@
         </is>
       </c>
       <c r="I139" t="n">
-        <v>28</v>
+        <v>50.90909090909091</v>
       </c>
       <c r="J139" t="n">
-        <v>17</v>
+        <v>56.66666666666666</v>
       </c>
     </row>
     <row r="140">
@@ -7134,10 +7134,10 @@
         </is>
       </c>
       <c r="I140" t="n">
-        <v>39</v>
+        <v>70.90909090909091</v>
       </c>
       <c r="J140" t="n">
-        <v>8</v>
+        <v>26.66666666666667</v>
       </c>
     </row>
     <row r="141">
@@ -7182,10 +7182,10 @@
         </is>
       </c>
       <c r="I141" t="n">
-        <v>35</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="J141" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="142">
@@ -7230,10 +7230,10 @@
         </is>
       </c>
       <c r="I142" t="n">
-        <v>30</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="J142" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="143">
@@ -7278,10 +7278,10 @@
         </is>
       </c>
       <c r="I143" t="n">
-        <v>36</v>
+        <v>65.45454545454545</v>
       </c>
       <c r="J143" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="144">
@@ -7326,10 +7326,10 @@
         </is>
       </c>
       <c r="I144" t="n">
-        <v>28</v>
+        <v>50.90909090909091</v>
       </c>
       <c r="J144" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="145">
@@ -7374,10 +7374,10 @@
         </is>
       </c>
       <c r="I145" t="n">
-        <v>32</v>
+        <v>58.18181818181818</v>
       </c>
       <c r="J145" t="n">
-        <v>16</v>
+        <v>53.33333333333334</v>
       </c>
     </row>
     <row r="146">
@@ -7422,10 +7422,10 @@
         </is>
       </c>
       <c r="I146" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J146" t="n">
-        <v>11</v>
+        <v>36.66666666666666</v>
       </c>
     </row>
     <row r="147">
@@ -7470,10 +7470,10 @@
         </is>
       </c>
       <c r="I147" t="n">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="J147" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="148">
@@ -7518,10 +7518,10 @@
         </is>
       </c>
       <c r="I148" t="n">
-        <v>28</v>
+        <v>50.90909090909091</v>
       </c>
       <c r="J148" t="n">
-        <v>11</v>
+        <v>36.66666666666666</v>
       </c>
     </row>
     <row r="149">
@@ -7566,10 +7566,10 @@
         </is>
       </c>
       <c r="I149" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J149" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="150">
@@ -7614,10 +7614,10 @@
         </is>
       </c>
       <c r="I150" t="n">
-        <v>27</v>
+        <v>49.09090909090909</v>
       </c>
       <c r="J150" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
     </row>
     <row r="151">
@@ -7662,10 +7662,10 @@
         </is>
       </c>
       <c r="I151" t="n">
-        <v>30</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="J151" t="n">
-        <v>27</v>
+        <v>90</v>
       </c>
     </row>
     <row r="152">
@@ -7710,10 +7710,10 @@
         </is>
       </c>
       <c r="I152" t="n">
-        <v>51</v>
+        <v>92.72727272727272</v>
       </c>
       <c r="J152" t="n">
-        <v>28</v>
+        <v>93.33333333333333</v>
       </c>
     </row>
     <row r="153">
@@ -7758,10 +7758,10 @@
         </is>
       </c>
       <c r="I153" t="n">
-        <v>48</v>
+        <v>87.27272727272727</v>
       </c>
       <c r="J153" t="n">
-        <v>13</v>
+        <v>43.33333333333334</v>
       </c>
     </row>
     <row r="154">
@@ -7806,10 +7806,10 @@
         </is>
       </c>
       <c r="I154" t="n">
-        <v>29</v>
+        <v>52.72727272727272</v>
       </c>
       <c r="J154" t="n">
-        <v>20</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="155">
@@ -7854,10 +7854,10 @@
         </is>
       </c>
       <c r="I155" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="J155" t="n">
-        <v>4</v>
+        <v>13.33333333333333</v>
       </c>
     </row>
     <row r="156">
@@ -7902,10 +7902,10 @@
         </is>
       </c>
       <c r="I156" t="n">
-        <v>21</v>
+        <v>38.18181818181819</v>
       </c>
       <c r="J156" t="n">
-        <v>20</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="157">
@@ -7950,10 +7950,10 @@
         </is>
       </c>
       <c r="I157" t="n">
-        <v>38</v>
+        <v>69.09090909090909</v>
       </c>
       <c r="J157" t="n">
-        <v>24</v>
+        <v>80</v>
       </c>
     </row>
     <row r="158">
@@ -7998,10 +7998,10 @@
         </is>
       </c>
       <c r="I158" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="J158" t="n">
-        <v>23</v>
+        <v>76.66666666666667</v>
       </c>
     </row>
     <row r="159">
@@ -8046,10 +8046,10 @@
         </is>
       </c>
       <c r="I159" t="n">
-        <v>23</v>
+        <v>41.81818181818181</v>
       </c>
       <c r="J159" t="n">
-        <v>13</v>
+        <v>43.33333333333334</v>
       </c>
     </row>
     <row r="160">
@@ -8094,10 +8094,10 @@
         </is>
       </c>
       <c r="I160" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J160" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="161">
@@ -8142,10 +8142,10 @@
         </is>
       </c>
       <c r="I161" t="n">
-        <v>26</v>
+        <v>47.27272727272727</v>
       </c>
       <c r="J161" t="n">
-        <v>16</v>
+        <v>53.33333333333334</v>
       </c>
     </row>
     <row r="162">
@@ -8190,10 +8190,10 @@
         </is>
       </c>
       <c r="I162" t="n">
-        <v>32</v>
+        <v>58.18181818181818</v>
       </c>
       <c r="J162" t="n">
-        <v>26</v>
+        <v>86.66666666666667</v>
       </c>
     </row>
     <row r="163">
@@ -8238,10 +8238,10 @@
         </is>
       </c>
       <c r="I163" t="n">
-        <v>42</v>
+        <v>76.36363636363637</v>
       </c>
       <c r="J163" t="n">
-        <v>20</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="164">
@@ -8286,10 +8286,10 @@
         </is>
       </c>
       <c r="I164" t="n">
-        <v>35</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="J164" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="165">
@@ -8334,10 +8334,10 @@
         </is>
       </c>
       <c r="I165" t="n">
-        <v>41</v>
+        <v>74.54545454545455</v>
       </c>
       <c r="J165" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="166">
@@ -8382,10 +8382,10 @@
         </is>
       </c>
       <c r="I166" t="n">
-        <v>43</v>
+        <v>78.18181818181819</v>
       </c>
       <c r="J166" t="n">
-        <v>25</v>
+        <v>83.33333333333334</v>
       </c>
     </row>
     <row r="167">
@@ -8430,10 +8430,10 @@
         </is>
       </c>
       <c r="I167" t="n">
-        <v>38</v>
+        <v>69.09090909090909</v>
       </c>
       <c r="J167" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="168">
@@ -8478,10 +8478,10 @@
         </is>
       </c>
       <c r="I168" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J168" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="169">
@@ -8526,10 +8526,10 @@
         </is>
       </c>
       <c r="I169" t="n">
-        <v>34</v>
+        <v>61.81818181818181</v>
       </c>
       <c r="J169" t="n">
-        <v>25</v>
+        <v>83.33333333333334</v>
       </c>
     </row>
     <row r="170">
@@ -8574,10 +8574,10 @@
         </is>
       </c>
       <c r="I170" t="n">
-        <v>35</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="J170" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="171">
@@ -8622,10 +8622,10 @@
         </is>
       </c>
       <c r="I171" t="n">
-        <v>17</v>
+        <v>30.90909090909091</v>
       </c>
       <c r="J171" t="n">
-        <v>10</v>
+        <v>33.33333333333333</v>
       </c>
     </row>
     <row r="172">
@@ -8670,10 +8670,10 @@
         </is>
       </c>
       <c r="I172" t="n">
-        <v>29</v>
+        <v>52.72727272727272</v>
       </c>
       <c r="J172" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="173">
@@ -8718,10 +8718,10 @@
         </is>
       </c>
       <c r="I173" t="n">
-        <v>29</v>
+        <v>52.72727272727272</v>
       </c>
       <c r="J173" t="n">
-        <v>19</v>
+        <v>63.33333333333333</v>
       </c>
     </row>
     <row r="174">
@@ -8766,10 +8766,10 @@
         </is>
       </c>
       <c r="I174" t="n">
-        <v>37</v>
+        <v>67.27272727272727</v>
       </c>
       <c r="J174" t="n">
-        <v>20</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="175">
@@ -8814,10 +8814,10 @@
         </is>
       </c>
       <c r="I175" t="n">
-        <v>30</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="J175" t="n">
-        <v>10</v>
+        <v>33.33333333333333</v>
       </c>
     </row>
     <row r="176">
@@ -8862,10 +8862,10 @@
         </is>
       </c>
       <c r="I176" t="n">
-        <v>49</v>
+        <v>89.09090909090909</v>
       </c>
       <c r="J176" t="n">
-        <v>28</v>
+        <v>93.33333333333333</v>
       </c>
     </row>
     <row r="177">
@@ -8910,10 +8910,10 @@
         </is>
       </c>
       <c r="I177" t="n">
-        <v>35</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="J177" t="n">
-        <v>25</v>
+        <v>83.33333333333334</v>
       </c>
     </row>
     <row r="178">
@@ -8958,10 +8958,10 @@
         </is>
       </c>
       <c r="I178" t="n">
-        <v>25</v>
+        <v>45.45454545454545</v>
       </c>
       <c r="J178" t="n">
-        <v>16</v>
+        <v>53.33333333333334</v>
       </c>
     </row>
     <row r="179">
@@ -9006,10 +9006,10 @@
         </is>
       </c>
       <c r="I179" t="n">
-        <v>29</v>
+        <v>52.72727272727272</v>
       </c>
       <c r="J179" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="180">
@@ -9054,10 +9054,10 @@
         </is>
       </c>
       <c r="I180" t="n">
-        <v>40</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="J180" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="181">
@@ -9102,10 +9102,10 @@
         </is>
       </c>
       <c r="I181" t="n">
-        <v>38</v>
+        <v>69.09090909090909</v>
       </c>
       <c r="J181" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="182">
@@ -9150,10 +9150,10 @@
         </is>
       </c>
       <c r="I182" t="n">
-        <v>29</v>
+        <v>52.72727272727272</v>
       </c>
       <c r="J182" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="183">
@@ -9198,10 +9198,10 @@
         </is>
       </c>
       <c r="I183" t="n">
-        <v>34</v>
+        <v>61.81818181818181</v>
       </c>
       <c r="J183" t="n">
-        <v>23</v>
+        <v>76.66666666666667</v>
       </c>
     </row>
     <row r="184">
@@ -9246,10 +9246,10 @@
         </is>
       </c>
       <c r="I184" t="n">
-        <v>45</v>
+        <v>81.81818181818183</v>
       </c>
       <c r="J184" t="n">
-        <v>23</v>
+        <v>76.66666666666667</v>
       </c>
     </row>
     <row r="185">
@@ -9294,10 +9294,10 @@
         </is>
       </c>
       <c r="I185" t="n">
-        <v>40</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="J185" t="n">
-        <v>14</v>
+        <v>46.66666666666666</v>
       </c>
     </row>
     <row r="186">
@@ -9342,10 +9342,10 @@
         </is>
       </c>
       <c r="I186" t="n">
-        <v>37</v>
+        <v>67.27272727272727</v>
       </c>
       <c r="J186" t="n">
-        <v>22</v>
+        <v>73.33333333333333</v>
       </c>
     </row>
     <row r="187">
@@ -9390,10 +9390,10 @@
         </is>
       </c>
       <c r="I187" t="n">
-        <v>31</v>
+        <v>56.36363636363636</v>
       </c>
       <c r="J187" t="n">
-        <v>14</v>
+        <v>46.66666666666666</v>
       </c>
     </row>
     <row r="188">
@@ -9438,10 +9438,10 @@
         </is>
       </c>
       <c r="I188" t="n">
-        <v>45</v>
+        <v>81.81818181818183</v>
       </c>
       <c r="J188" t="n">
-        <v>28</v>
+        <v>93.33333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Mantener columnas de índices originales junto con las normalizadas para evitar errores en Power BI
</commit_message>
<xml_diff>
--- a/output/df_docentes_final.xlsx
+++ b/output/df_docentes_final.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J188"/>
+  <dimension ref="A1:L188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,10 +459,20 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>Indice_Conocimiento</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>Indice_Conocimiento_Norm</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Indice_Capacidades_Respuesta</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
         <is>
           <t>Indice_Capacidades_Respuesta_Norm</t>
         </is>
@@ -510,9 +520,15 @@
         </is>
       </c>
       <c r="I2" t="n">
+        <v>46</v>
+      </c>
+      <c r="J2" t="n">
         <v>83.63636363636363</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
+        <v>30</v>
+      </c>
+      <c r="L2" t="n">
         <v>100</v>
       </c>
     </row>
@@ -558,9 +574,15 @@
         </is>
       </c>
       <c r="I3" t="n">
+        <v>30</v>
+      </c>
+      <c r="J3" t="n">
         <v>54.54545454545454</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
+        <v>23</v>
+      </c>
+      <c r="L3" t="n">
         <v>76.66666666666667</v>
       </c>
     </row>
@@ -606,9 +628,15 @@
         </is>
       </c>
       <c r="I4" t="n">
+        <v>27</v>
+      </c>
+      <c r="J4" t="n">
         <v>49.09090909090909</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L4" t="n">
         <v>16.66666666666666</v>
       </c>
     </row>
@@ -654,9 +682,15 @@
         </is>
       </c>
       <c r="I5" t="n">
+        <v>49</v>
+      </c>
+      <c r="J5" t="n">
         <v>89.09090909090909</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
+        <v>29</v>
+      </c>
+      <c r="L5" t="n">
         <v>96.66666666666667</v>
       </c>
     </row>
@@ -702,9 +736,15 @@
         </is>
       </c>
       <c r="I6" t="n">
+        <v>28</v>
+      </c>
+      <c r="J6" t="n">
         <v>50.90909090909091</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
+        <v>15</v>
+      </c>
+      <c r="L6" t="n">
         <v>50</v>
       </c>
     </row>
@@ -750,9 +790,15 @@
         </is>
       </c>
       <c r="I7" t="n">
+        <v>27</v>
+      </c>
+      <c r="J7" t="n">
         <v>49.09090909090909</v>
       </c>
-      <c r="J7" t="n">
+      <c r="K7" t="n">
+        <v>22</v>
+      </c>
+      <c r="L7" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -798,9 +844,15 @@
         </is>
       </c>
       <c r="I8" t="n">
+        <v>28</v>
+      </c>
+      <c r="J8" t="n">
         <v>50.90909090909091</v>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
+        <v>18</v>
+      </c>
+      <c r="L8" t="n">
         <v>60</v>
       </c>
     </row>
@@ -846,9 +898,15 @@
         </is>
       </c>
       <c r="I9" t="n">
+        <v>29</v>
+      </c>
+      <c r="J9" t="n">
         <v>52.72727272727272</v>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
+        <v>22</v>
+      </c>
+      <c r="L9" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -894,9 +952,15 @@
         </is>
       </c>
       <c r="I10" t="n">
+        <v>35</v>
+      </c>
+      <c r="J10" t="n">
         <v>63.63636363636363</v>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
+        <v>11</v>
+      </c>
+      <c r="L10" t="n">
         <v>36.66666666666666</v>
       </c>
     </row>
@@ -942,9 +1006,15 @@
         </is>
       </c>
       <c r="I11" t="n">
+        <v>32</v>
+      </c>
+      <c r="J11" t="n">
         <v>58.18181818181818</v>
       </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
+        <v>21</v>
+      </c>
+      <c r="L11" t="n">
         <v>70</v>
       </c>
     </row>
@@ -990,11 +1060,17 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>60</v>
+        <v>33</v>
       </c>
       <c r="J12" t="n">
         <v>60</v>
       </c>
+      <c r="K12" t="n">
+        <v>18</v>
+      </c>
+      <c r="L12" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1038,9 +1114,15 @@
         </is>
       </c>
       <c r="I13" t="n">
+        <v>26</v>
+      </c>
+      <c r="J13" t="n">
         <v>47.27272727272727</v>
       </c>
-      <c r="J13" t="n">
+      <c r="K13" t="n">
+        <v>20</v>
+      </c>
+      <c r="L13" t="n">
         <v>66.66666666666666</v>
       </c>
     </row>
@@ -1086,9 +1168,15 @@
         </is>
       </c>
       <c r="I14" t="n">
+        <v>31</v>
+      </c>
+      <c r="J14" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J14" t="n">
+      <c r="K14" t="n">
+        <v>16</v>
+      </c>
+      <c r="L14" t="n">
         <v>53.33333333333334</v>
       </c>
     </row>
@@ -1134,9 +1222,15 @@
         </is>
       </c>
       <c r="I15" t="n">
+        <v>34</v>
+      </c>
+      <c r="J15" t="n">
         <v>61.81818181818181</v>
       </c>
-      <c r="J15" t="n">
+      <c r="K15" t="n">
+        <v>9</v>
+      </c>
+      <c r="L15" t="n">
         <v>30</v>
       </c>
     </row>
@@ -1182,9 +1276,15 @@
         </is>
       </c>
       <c r="I16" t="n">
+        <v>36</v>
+      </c>
+      <c r="J16" t="n">
         <v>65.45454545454545</v>
       </c>
-      <c r="J16" t="n">
+      <c r="K16" t="n">
+        <v>18</v>
+      </c>
+      <c r="L16" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1230,9 +1330,15 @@
         </is>
       </c>
       <c r="I17" t="n">
+        <v>30</v>
+      </c>
+      <c r="J17" t="n">
         <v>54.54545454545454</v>
       </c>
-      <c r="J17" t="n">
+      <c r="K17" t="n">
+        <v>19</v>
+      </c>
+      <c r="L17" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -1278,9 +1384,15 @@
         </is>
       </c>
       <c r="I18" t="n">
+        <v>24</v>
+      </c>
+      <c r="J18" t="n">
         <v>43.63636363636363</v>
       </c>
-      <c r="J18" t="n">
+      <c r="K18" t="n">
+        <v>20</v>
+      </c>
+      <c r="L18" t="n">
         <v>66.66666666666666</v>
       </c>
     </row>
@@ -1326,9 +1438,15 @@
         </is>
       </c>
       <c r="I19" t="n">
+        <v>37</v>
+      </c>
+      <c r="J19" t="n">
         <v>67.27272727272727</v>
       </c>
-      <c r="J19" t="n">
+      <c r="K19" t="n">
+        <v>19</v>
+      </c>
+      <c r="L19" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -1374,9 +1492,15 @@
         </is>
       </c>
       <c r="I20" t="n">
+        <v>30</v>
+      </c>
+      <c r="J20" t="n">
         <v>54.54545454545454</v>
       </c>
-      <c r="J20" t="n">
+      <c r="K20" t="n">
+        <v>18</v>
+      </c>
+      <c r="L20" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1422,9 +1546,15 @@
         </is>
       </c>
       <c r="I21" t="n">
+        <v>39</v>
+      </c>
+      <c r="J21" t="n">
         <v>70.90909090909091</v>
       </c>
-      <c r="J21" t="n">
+      <c r="K21" t="n">
+        <v>19</v>
+      </c>
+      <c r="L21" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -1470,9 +1600,15 @@
         </is>
       </c>
       <c r="I22" t="n">
+        <v>19</v>
+      </c>
+      <c r="J22" t="n">
         <v>34.54545454545455</v>
       </c>
-      <c r="J22" t="n">
+      <c r="K22" t="n">
+        <v>11</v>
+      </c>
+      <c r="L22" t="n">
         <v>36.66666666666666</v>
       </c>
     </row>
@@ -1518,9 +1654,15 @@
         </is>
       </c>
       <c r="I23" t="n">
+        <v>45</v>
+      </c>
+      <c r="J23" t="n">
         <v>81.81818181818183</v>
       </c>
-      <c r="J23" t="n">
+      <c r="K23" t="n">
+        <v>15</v>
+      </c>
+      <c r="L23" t="n">
         <v>50</v>
       </c>
     </row>
@@ -1566,9 +1708,15 @@
         </is>
       </c>
       <c r="I24" t="n">
+        <v>27</v>
+      </c>
+      <c r="J24" t="n">
         <v>49.09090909090909</v>
       </c>
-      <c r="J24" t="n">
+      <c r="K24" t="n">
+        <v>22</v>
+      </c>
+      <c r="L24" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -1614,9 +1762,15 @@
         </is>
       </c>
       <c r="I25" t="n">
+        <v>35</v>
+      </c>
+      <c r="J25" t="n">
         <v>63.63636363636363</v>
       </c>
-      <c r="J25" t="n">
+      <c r="K25" t="n">
+        <v>11</v>
+      </c>
+      <c r="L25" t="n">
         <v>36.66666666666666</v>
       </c>
     </row>
@@ -1662,9 +1816,15 @@
         </is>
       </c>
       <c r="I26" t="n">
+        <v>32</v>
+      </c>
+      <c r="J26" t="n">
         <v>58.18181818181818</v>
       </c>
-      <c r="J26" t="n">
+      <c r="K26" t="n">
+        <v>20</v>
+      </c>
+      <c r="L26" t="n">
         <v>66.66666666666666</v>
       </c>
     </row>
@@ -1710,9 +1870,15 @@
         </is>
       </c>
       <c r="I27" t="n">
+        <v>40</v>
+      </c>
+      <c r="J27" t="n">
         <v>72.72727272727273</v>
       </c>
-      <c r="J27" t="n">
+      <c r="K27" t="n">
+        <v>26</v>
+      </c>
+      <c r="L27" t="n">
         <v>86.66666666666667</v>
       </c>
     </row>
@@ -1758,9 +1924,15 @@
         </is>
       </c>
       <c r="I28" t="n">
+        <v>33</v>
+      </c>
+      <c r="J28" t="n">
         <v>60</v>
       </c>
-      <c r="J28" t="n">
+      <c r="K28" t="n">
+        <v>22</v>
+      </c>
+      <c r="L28" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -1806,9 +1978,15 @@
         </is>
       </c>
       <c r="I29" t="n">
+        <v>32</v>
+      </c>
+      <c r="J29" t="n">
         <v>58.18181818181818</v>
       </c>
-      <c r="J29" t="n">
+      <c r="K29" t="n">
+        <v>18</v>
+      </c>
+      <c r="L29" t="n">
         <v>60</v>
       </c>
     </row>
@@ -1854,9 +2032,15 @@
         </is>
       </c>
       <c r="I30" t="n">
+        <v>27</v>
+      </c>
+      <c r="J30" t="n">
         <v>49.09090909090909</v>
       </c>
-      <c r="J30" t="n">
+      <c r="K30" t="n">
+        <v>14</v>
+      </c>
+      <c r="L30" t="n">
         <v>46.66666666666666</v>
       </c>
     </row>
@@ -1902,9 +2086,15 @@
         </is>
       </c>
       <c r="I31" t="n">
+        <v>36</v>
+      </c>
+      <c r="J31" t="n">
         <v>65.45454545454545</v>
       </c>
-      <c r="J31" t="n">
+      <c r="K31" t="n">
+        <v>21</v>
+      </c>
+      <c r="L31" t="n">
         <v>70</v>
       </c>
     </row>
@@ -1950,9 +2140,15 @@
         </is>
       </c>
       <c r="I32" t="n">
+        <v>39</v>
+      </c>
+      <c r="J32" t="n">
         <v>70.90909090909091</v>
       </c>
-      <c r="J32" t="n">
+      <c r="K32" t="n">
+        <v>14</v>
+      </c>
+      <c r="L32" t="n">
         <v>46.66666666666666</v>
       </c>
     </row>
@@ -1998,9 +2194,15 @@
         </is>
       </c>
       <c r="I33" t="n">
+        <v>36</v>
+      </c>
+      <c r="J33" t="n">
         <v>65.45454545454545</v>
       </c>
-      <c r="J33" t="n">
+      <c r="K33" t="n">
+        <v>8</v>
+      </c>
+      <c r="L33" t="n">
         <v>26.66666666666667</v>
       </c>
     </row>
@@ -2046,9 +2248,15 @@
         </is>
       </c>
       <c r="I34" t="n">
+        <v>39</v>
+      </c>
+      <c r="J34" t="n">
         <v>70.90909090909091</v>
       </c>
-      <c r="J34" t="n">
+      <c r="K34" t="n">
+        <v>19</v>
+      </c>
+      <c r="L34" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -2094,9 +2302,15 @@
         </is>
       </c>
       <c r="I35" t="n">
+        <v>35</v>
+      </c>
+      <c r="J35" t="n">
         <v>63.63636363636363</v>
       </c>
-      <c r="J35" t="n">
+      <c r="K35" t="n">
+        <v>15</v>
+      </c>
+      <c r="L35" t="n">
         <v>50</v>
       </c>
     </row>
@@ -2142,9 +2356,15 @@
         </is>
       </c>
       <c r="I36" t="n">
+        <v>33</v>
+      </c>
+      <c r="J36" t="n">
         <v>60</v>
       </c>
-      <c r="J36" t="n">
+      <c r="K36" t="n">
+        <v>21</v>
+      </c>
+      <c r="L36" t="n">
         <v>70</v>
       </c>
     </row>
@@ -2190,9 +2410,15 @@
         </is>
       </c>
       <c r="I37" t="n">
+        <v>32</v>
+      </c>
+      <c r="J37" t="n">
         <v>58.18181818181818</v>
       </c>
-      <c r="J37" t="n">
+      <c r="K37" t="n">
+        <v>15</v>
+      </c>
+      <c r="L37" t="n">
         <v>50</v>
       </c>
     </row>
@@ -2238,9 +2464,15 @@
         </is>
       </c>
       <c r="I38" t="n">
+        <v>24</v>
+      </c>
+      <c r="J38" t="n">
         <v>43.63636363636363</v>
       </c>
-      <c r="J38" t="n">
+      <c r="K38" t="n">
+        <v>23</v>
+      </c>
+      <c r="L38" t="n">
         <v>76.66666666666667</v>
       </c>
     </row>
@@ -2286,9 +2518,15 @@
         </is>
       </c>
       <c r="I39" t="n">
+        <v>29</v>
+      </c>
+      <c r="J39" t="n">
         <v>52.72727272727272</v>
       </c>
-      <c r="J39" t="n">
+      <c r="K39" t="n">
+        <v>15</v>
+      </c>
+      <c r="L39" t="n">
         <v>50</v>
       </c>
     </row>
@@ -2334,9 +2572,15 @@
         </is>
       </c>
       <c r="I40" t="n">
+        <v>41</v>
+      </c>
+      <c r="J40" t="n">
         <v>74.54545454545455</v>
       </c>
-      <c r="J40" t="n">
+      <c r="K40" t="n">
+        <v>22</v>
+      </c>
+      <c r="L40" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -2382,9 +2626,15 @@
         </is>
       </c>
       <c r="I41" t="n">
+        <v>38</v>
+      </c>
+      <c r="J41" t="n">
         <v>69.09090909090909</v>
       </c>
-      <c r="J41" t="n">
+      <c r="K41" t="n">
+        <v>20</v>
+      </c>
+      <c r="L41" t="n">
         <v>66.66666666666666</v>
       </c>
     </row>
@@ -2430,9 +2680,15 @@
         </is>
       </c>
       <c r="I42" t="n">
+        <v>49</v>
+      </c>
+      <c r="J42" t="n">
         <v>89.09090909090909</v>
       </c>
-      <c r="J42" t="n">
+      <c r="K42" t="n">
+        <v>26</v>
+      </c>
+      <c r="L42" t="n">
         <v>86.66666666666667</v>
       </c>
     </row>
@@ -2478,9 +2734,15 @@
         </is>
       </c>
       <c r="I43" t="n">
+        <v>41</v>
+      </c>
+      <c r="J43" t="n">
         <v>74.54545454545455</v>
       </c>
-      <c r="J43" t="n">
+      <c r="K43" t="n">
+        <v>22</v>
+      </c>
+      <c r="L43" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -2526,9 +2788,15 @@
         </is>
       </c>
       <c r="I44" t="n">
+        <v>33</v>
+      </c>
+      <c r="J44" t="n">
         <v>60</v>
       </c>
-      <c r="J44" t="n">
+      <c r="K44" t="n">
+        <v>21</v>
+      </c>
+      <c r="L44" t="n">
         <v>70</v>
       </c>
     </row>
@@ -2574,9 +2842,15 @@
         </is>
       </c>
       <c r="I45" t="n">
+        <v>42</v>
+      </c>
+      <c r="J45" t="n">
         <v>76.36363636363637</v>
       </c>
-      <c r="J45" t="n">
+      <c r="K45" t="n">
+        <v>13</v>
+      </c>
+      <c r="L45" t="n">
         <v>43.33333333333334</v>
       </c>
     </row>
@@ -2622,9 +2896,15 @@
         </is>
       </c>
       <c r="I46" t="n">
+        <v>30</v>
+      </c>
+      <c r="J46" t="n">
         <v>54.54545454545454</v>
       </c>
-      <c r="J46" t="n">
+      <c r="K46" t="n">
+        <v>8</v>
+      </c>
+      <c r="L46" t="n">
         <v>26.66666666666667</v>
       </c>
     </row>
@@ -2670,9 +2950,15 @@
         </is>
       </c>
       <c r="I47" t="n">
+        <v>37</v>
+      </c>
+      <c r="J47" t="n">
         <v>67.27272727272727</v>
       </c>
-      <c r="J47" t="n">
+      <c r="K47" t="n">
+        <v>20</v>
+      </c>
+      <c r="L47" t="n">
         <v>66.66666666666666</v>
       </c>
     </row>
@@ -2718,9 +3004,15 @@
         </is>
       </c>
       <c r="I48" t="n">
+        <v>53</v>
+      </c>
+      <c r="J48" t="n">
         <v>96.36363636363636</v>
       </c>
-      <c r="J48" t="n">
+      <c r="K48" t="n">
+        <v>20</v>
+      </c>
+      <c r="L48" t="n">
         <v>66.66666666666666</v>
       </c>
     </row>
@@ -2766,9 +3058,15 @@
         </is>
       </c>
       <c r="I49" t="n">
+        <v>38</v>
+      </c>
+      <c r="J49" t="n">
         <v>69.09090909090909</v>
       </c>
-      <c r="J49" t="n">
+      <c r="K49" t="n">
+        <v>20</v>
+      </c>
+      <c r="L49" t="n">
         <v>66.66666666666666</v>
       </c>
     </row>
@@ -2814,9 +3112,15 @@
         </is>
       </c>
       <c r="I50" t="n">
+        <v>31</v>
+      </c>
+      <c r="J50" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J50" t="n">
+      <c r="K50" t="n">
+        <v>17</v>
+      </c>
+      <c r="L50" t="n">
         <v>56.66666666666666</v>
       </c>
     </row>
@@ -2862,9 +3166,15 @@
         </is>
       </c>
       <c r="I51" t="n">
+        <v>25</v>
+      </c>
+      <c r="J51" t="n">
         <v>45.45454545454545</v>
       </c>
-      <c r="J51" t="n">
+      <c r="K51" t="n">
+        <v>25</v>
+      </c>
+      <c r="L51" t="n">
         <v>83.33333333333334</v>
       </c>
     </row>
@@ -2910,9 +3220,15 @@
         </is>
       </c>
       <c r="I52" t="n">
+        <v>37</v>
+      </c>
+      <c r="J52" t="n">
         <v>67.27272727272727</v>
       </c>
-      <c r="J52" t="n">
+      <c r="K52" t="n">
+        <v>18</v>
+      </c>
+      <c r="L52" t="n">
         <v>60</v>
       </c>
     </row>
@@ -2958,9 +3274,15 @@
         </is>
       </c>
       <c r="I53" t="n">
+        <v>31</v>
+      </c>
+      <c r="J53" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J53" t="n">
+      <c r="K53" t="n">
+        <v>20</v>
+      </c>
+      <c r="L53" t="n">
         <v>66.66666666666666</v>
       </c>
     </row>
@@ -3006,9 +3328,15 @@
         </is>
       </c>
       <c r="I54" t="n">
+        <v>42</v>
+      </c>
+      <c r="J54" t="n">
         <v>76.36363636363637</v>
       </c>
-      <c r="J54" t="n">
+      <c r="K54" t="n">
+        <v>19</v>
+      </c>
+      <c r="L54" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -3054,9 +3382,15 @@
         </is>
       </c>
       <c r="I55" t="n">
+        <v>37</v>
+      </c>
+      <c r="J55" t="n">
         <v>67.27272727272727</v>
       </c>
-      <c r="J55" t="n">
+      <c r="K55" t="n">
+        <v>22</v>
+      </c>
+      <c r="L55" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -3102,9 +3436,15 @@
         </is>
       </c>
       <c r="I56" t="n">
+        <v>32</v>
+      </c>
+      <c r="J56" t="n">
         <v>58.18181818181818</v>
       </c>
-      <c r="J56" t="n">
+      <c r="K56" t="n">
+        <v>14</v>
+      </c>
+      <c r="L56" t="n">
         <v>46.66666666666666</v>
       </c>
     </row>
@@ -3150,9 +3490,15 @@
         </is>
       </c>
       <c r="I57" t="n">
+        <v>14</v>
+      </c>
+      <c r="J57" t="n">
         <v>25.45454545454545</v>
       </c>
-      <c r="J57" t="n">
+      <c r="K57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3198,9 +3544,15 @@
         </is>
       </c>
       <c r="I58" t="n">
+        <v>49</v>
+      </c>
+      <c r="J58" t="n">
         <v>89.09090909090909</v>
       </c>
-      <c r="J58" t="n">
+      <c r="K58" t="n">
+        <v>19</v>
+      </c>
+      <c r="L58" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -3246,9 +3598,15 @@
         </is>
       </c>
       <c r="I59" t="n">
+        <v>27</v>
+      </c>
+      <c r="J59" t="n">
         <v>49.09090909090909</v>
       </c>
-      <c r="J59" t="n">
+      <c r="K59" t="n">
+        <v>13</v>
+      </c>
+      <c r="L59" t="n">
         <v>43.33333333333334</v>
       </c>
     </row>
@@ -3294,9 +3652,15 @@
         </is>
       </c>
       <c r="I60" t="n">
+        <v>46</v>
+      </c>
+      <c r="J60" t="n">
         <v>83.63636363636363</v>
       </c>
-      <c r="J60" t="n">
+      <c r="K60" t="n">
+        <v>23</v>
+      </c>
+      <c r="L60" t="n">
         <v>76.66666666666667</v>
       </c>
     </row>
@@ -3342,9 +3706,15 @@
         </is>
       </c>
       <c r="I61" t="n">
+        <v>33</v>
+      </c>
+      <c r="J61" t="n">
         <v>60</v>
       </c>
-      <c r="J61" t="n">
+      <c r="K61" t="n">
+        <v>13</v>
+      </c>
+      <c r="L61" t="n">
         <v>43.33333333333334</v>
       </c>
     </row>
@@ -3390,9 +3760,15 @@
         </is>
       </c>
       <c r="I62" t="n">
+        <v>37</v>
+      </c>
+      <c r="J62" t="n">
         <v>67.27272727272727</v>
       </c>
-      <c r="J62" t="n">
+      <c r="K62" t="n">
+        <v>28</v>
+      </c>
+      <c r="L62" t="n">
         <v>93.33333333333333</v>
       </c>
     </row>
@@ -3438,9 +3814,15 @@
         </is>
       </c>
       <c r="I63" t="n">
+        <v>37</v>
+      </c>
+      <c r="J63" t="n">
         <v>67.27272727272727</v>
       </c>
-      <c r="J63" t="n">
+      <c r="K63" t="n">
+        <v>13</v>
+      </c>
+      <c r="L63" t="n">
         <v>43.33333333333334</v>
       </c>
     </row>
@@ -3486,9 +3868,15 @@
         </is>
       </c>
       <c r="I64" t="n">
+        <v>42</v>
+      </c>
+      <c r="J64" t="n">
         <v>76.36363636363637</v>
       </c>
-      <c r="J64" t="n">
+      <c r="K64" t="n">
+        <v>22</v>
+      </c>
+      <c r="L64" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -3534,9 +3922,15 @@
         </is>
       </c>
       <c r="I65" t="n">
+        <v>33</v>
+      </c>
+      <c r="J65" t="n">
         <v>60</v>
       </c>
-      <c r="J65" t="n">
+      <c r="K65" t="n">
+        <v>9</v>
+      </c>
+      <c r="L65" t="n">
         <v>30</v>
       </c>
     </row>
@@ -3582,9 +3976,15 @@
         </is>
       </c>
       <c r="I66" t="n">
+        <v>30</v>
+      </c>
+      <c r="J66" t="n">
         <v>54.54545454545454</v>
       </c>
-      <c r="J66" t="n">
+      <c r="K66" t="n">
+        <v>12</v>
+      </c>
+      <c r="L66" t="n">
         <v>40</v>
       </c>
     </row>
@@ -3630,9 +4030,15 @@
         </is>
       </c>
       <c r="I67" t="n">
+        <v>33</v>
+      </c>
+      <c r="J67" t="n">
         <v>60</v>
       </c>
-      <c r="J67" t="n">
+      <c r="K67" t="n">
+        <v>1</v>
+      </c>
+      <c r="L67" t="n">
         <v>3.333333333333333</v>
       </c>
     </row>
@@ -3678,9 +4084,15 @@
         </is>
       </c>
       <c r="I68" t="n">
+        <v>29</v>
+      </c>
+      <c r="J68" t="n">
         <v>52.72727272727272</v>
       </c>
-      <c r="J68" t="n">
+      <c r="K68" t="n">
+        <v>22</v>
+      </c>
+      <c r="L68" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -3726,9 +4138,15 @@
         </is>
       </c>
       <c r="I69" t="n">
+        <v>31</v>
+      </c>
+      <c r="J69" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J69" t="n">
+      <c r="K69" t="n">
+        <v>14</v>
+      </c>
+      <c r="L69" t="n">
         <v>46.66666666666666</v>
       </c>
     </row>
@@ -3774,9 +4192,15 @@
         </is>
       </c>
       <c r="I70" t="n">
+        <v>30</v>
+      </c>
+      <c r="J70" t="n">
         <v>54.54545454545454</v>
       </c>
-      <c r="J70" t="n">
+      <c r="K70" t="n">
+        <v>19</v>
+      </c>
+      <c r="L70" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -3822,9 +4246,15 @@
         </is>
       </c>
       <c r="I71" t="n">
+        <v>55</v>
+      </c>
+      <c r="J71" t="n">
         <v>100</v>
       </c>
-      <c r="J71" t="n">
+      <c r="K71" t="n">
+        <v>25</v>
+      </c>
+      <c r="L71" t="n">
         <v>83.33333333333334</v>
       </c>
     </row>
@@ -3870,9 +4300,15 @@
         </is>
       </c>
       <c r="I72" t="n">
+        <v>39</v>
+      </c>
+      <c r="J72" t="n">
         <v>70.90909090909091</v>
       </c>
-      <c r="J72" t="n">
+      <c r="K72" t="n">
+        <v>26</v>
+      </c>
+      <c r="L72" t="n">
         <v>86.66666666666667</v>
       </c>
     </row>
@@ -3918,9 +4354,15 @@
         </is>
       </c>
       <c r="I73" t="n">
+        <v>25</v>
+      </c>
+      <c r="J73" t="n">
         <v>45.45454545454545</v>
       </c>
-      <c r="J73" t="n">
+      <c r="K73" t="n">
+        <v>21</v>
+      </c>
+      <c r="L73" t="n">
         <v>70</v>
       </c>
     </row>
@@ -3966,9 +4408,15 @@
         </is>
       </c>
       <c r="I74" t="n">
+        <v>25</v>
+      </c>
+      <c r="J74" t="n">
         <v>45.45454545454545</v>
       </c>
-      <c r="J74" t="n">
+      <c r="K74" t="n">
+        <v>11</v>
+      </c>
+      <c r="L74" t="n">
         <v>36.66666666666666</v>
       </c>
     </row>
@@ -4014,9 +4462,15 @@
         </is>
       </c>
       <c r="I75" t="n">
+        <v>41</v>
+      </c>
+      <c r="J75" t="n">
         <v>74.54545454545455</v>
       </c>
-      <c r="J75" t="n">
+      <c r="K75" t="n">
+        <v>30</v>
+      </c>
+      <c r="L75" t="n">
         <v>100</v>
       </c>
     </row>
@@ -4062,9 +4516,15 @@
         </is>
       </c>
       <c r="I76" t="n">
+        <v>32</v>
+      </c>
+      <c r="J76" t="n">
         <v>58.18181818181818</v>
       </c>
-      <c r="J76" t="n">
+      <c r="K76" t="n">
+        <v>19</v>
+      </c>
+      <c r="L76" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -4110,9 +4570,15 @@
         </is>
       </c>
       <c r="I77" t="n">
+        <v>44</v>
+      </c>
+      <c r="J77" t="n">
         <v>80</v>
       </c>
-      <c r="J77" t="n">
+      <c r="K77" t="n">
+        <v>25</v>
+      </c>
+      <c r="L77" t="n">
         <v>83.33333333333334</v>
       </c>
     </row>
@@ -4158,9 +4624,15 @@
         </is>
       </c>
       <c r="I78" t="n">
+        <v>28</v>
+      </c>
+      <c r="J78" t="n">
         <v>50.90909090909091</v>
       </c>
-      <c r="J78" t="n">
+      <c r="K78" t="n">
+        <v>21</v>
+      </c>
+      <c r="L78" t="n">
         <v>70</v>
       </c>
     </row>
@@ -4206,9 +4678,15 @@
         </is>
       </c>
       <c r="I79" t="n">
+        <v>31</v>
+      </c>
+      <c r="J79" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J79" t="n">
+      <c r="K79" t="n">
+        <v>16</v>
+      </c>
+      <c r="L79" t="n">
         <v>53.33333333333334</v>
       </c>
     </row>
@@ -4254,9 +4732,15 @@
         </is>
       </c>
       <c r="I80" t="n">
+        <v>30</v>
+      </c>
+      <c r="J80" t="n">
         <v>54.54545454545454</v>
       </c>
-      <c r="J80" t="n">
+      <c r="K80" t="n">
+        <v>16</v>
+      </c>
+      <c r="L80" t="n">
         <v>53.33333333333334</v>
       </c>
     </row>
@@ -4302,9 +4786,15 @@
         </is>
       </c>
       <c r="I81" t="n">
+        <v>31</v>
+      </c>
+      <c r="J81" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J81" t="n">
+      <c r="K81" t="n">
+        <v>19</v>
+      </c>
+      <c r="L81" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -4350,9 +4840,15 @@
         </is>
       </c>
       <c r="I82" t="n">
+        <v>36</v>
+      </c>
+      <c r="J82" t="n">
         <v>65.45454545454545</v>
       </c>
-      <c r="J82" t="n">
+      <c r="K82" t="n">
+        <v>18</v>
+      </c>
+      <c r="L82" t="n">
         <v>60</v>
       </c>
     </row>
@@ -4398,9 +4894,15 @@
         </is>
       </c>
       <c r="I83" t="n">
+        <v>38</v>
+      </c>
+      <c r="J83" t="n">
         <v>69.09090909090909</v>
       </c>
-      <c r="J83" t="n">
+      <c r="K83" t="n">
+        <v>18</v>
+      </c>
+      <c r="L83" t="n">
         <v>60</v>
       </c>
     </row>
@@ -4446,9 +4948,15 @@
         </is>
       </c>
       <c r="I84" t="n">
+        <v>31</v>
+      </c>
+      <c r="J84" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J84" t="n">
+      <c r="K84" t="n">
+        <v>10</v>
+      </c>
+      <c r="L84" t="n">
         <v>33.33333333333333</v>
       </c>
     </row>
@@ -4494,9 +5002,15 @@
         </is>
       </c>
       <c r="I85" t="n">
+        <v>40</v>
+      </c>
+      <c r="J85" t="n">
         <v>72.72727272727273</v>
       </c>
-      <c r="J85" t="n">
+      <c r="K85" t="n">
+        <v>22</v>
+      </c>
+      <c r="L85" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -4542,9 +5056,15 @@
         </is>
       </c>
       <c r="I86" t="n">
+        <v>36</v>
+      </c>
+      <c r="J86" t="n">
         <v>65.45454545454545</v>
       </c>
-      <c r="J86" t="n">
+      <c r="K86" t="n">
+        <v>23</v>
+      </c>
+      <c r="L86" t="n">
         <v>76.66666666666667</v>
       </c>
     </row>
@@ -4590,9 +5110,15 @@
         </is>
       </c>
       <c r="I87" t="n">
+        <v>31</v>
+      </c>
+      <c r="J87" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J87" t="n">
+      <c r="K87" t="n">
+        <v>7</v>
+      </c>
+      <c r="L87" t="n">
         <v>23.33333333333333</v>
       </c>
     </row>
@@ -4638,9 +5164,15 @@
         </is>
       </c>
       <c r="I88" t="n">
+        <v>39</v>
+      </c>
+      <c r="J88" t="n">
         <v>70.90909090909091</v>
       </c>
-      <c r="J88" t="n">
+      <c r="K88" t="n">
+        <v>19</v>
+      </c>
+      <c r="L88" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -4686,9 +5218,15 @@
         </is>
       </c>
       <c r="I89" t="n">
+        <v>13</v>
+      </c>
+      <c r="J89" t="n">
         <v>23.63636363636364</v>
       </c>
-      <c r="J89" t="n">
+      <c r="K89" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4734,9 +5272,15 @@
         </is>
       </c>
       <c r="I90" t="n">
+        <v>32</v>
+      </c>
+      <c r="J90" t="n">
         <v>58.18181818181818</v>
       </c>
-      <c r="J90" t="n">
+      <c r="K90" t="n">
+        <v>22</v>
+      </c>
+      <c r="L90" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -4782,9 +5326,15 @@
         </is>
       </c>
       <c r="I91" t="n">
+        <v>39</v>
+      </c>
+      <c r="J91" t="n">
         <v>70.90909090909091</v>
       </c>
-      <c r="J91" t="n">
+      <c r="K91" t="n">
+        <v>26</v>
+      </c>
+      <c r="L91" t="n">
         <v>86.66666666666667</v>
       </c>
     </row>
@@ -4830,9 +5380,15 @@
         </is>
       </c>
       <c r="I92" t="n">
+        <v>35</v>
+      </c>
+      <c r="J92" t="n">
         <v>63.63636363636363</v>
       </c>
-      <c r="J92" t="n">
+      <c r="K92" t="n">
+        <v>18</v>
+      </c>
+      <c r="L92" t="n">
         <v>60</v>
       </c>
     </row>
@@ -4878,9 +5434,15 @@
         </is>
       </c>
       <c r="I93" t="n">
+        <v>26</v>
+      </c>
+      <c r="J93" t="n">
         <v>47.27272727272727</v>
       </c>
-      <c r="J93" t="n">
+      <c r="K93" t="n">
+        <v>6</v>
+      </c>
+      <c r="L93" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4926,9 +5488,15 @@
         </is>
       </c>
       <c r="I94" t="n">
+        <v>29</v>
+      </c>
+      <c r="J94" t="n">
         <v>52.72727272727272</v>
       </c>
-      <c r="J94" t="n">
+      <c r="K94" t="n">
+        <v>13</v>
+      </c>
+      <c r="L94" t="n">
         <v>43.33333333333334</v>
       </c>
     </row>
@@ -4974,9 +5542,15 @@
         </is>
       </c>
       <c r="I95" t="n">
+        <v>32</v>
+      </c>
+      <c r="J95" t="n">
         <v>58.18181818181818</v>
       </c>
-      <c r="J95" t="n">
+      <c r="K95" t="n">
+        <v>13</v>
+      </c>
+      <c r="L95" t="n">
         <v>43.33333333333334</v>
       </c>
     </row>
@@ -5022,9 +5596,15 @@
         </is>
       </c>
       <c r="I96" t="n">
+        <v>41</v>
+      </c>
+      <c r="J96" t="n">
         <v>74.54545454545455</v>
       </c>
-      <c r="J96" t="n">
+      <c r="K96" t="n">
+        <v>18</v>
+      </c>
+      <c r="L96" t="n">
         <v>60</v>
       </c>
     </row>
@@ -5070,9 +5650,15 @@
         </is>
       </c>
       <c r="I97" t="n">
+        <v>33</v>
+      </c>
+      <c r="J97" t="n">
         <v>60</v>
       </c>
-      <c r="J97" t="n">
+      <c r="K97" t="n">
+        <v>10</v>
+      </c>
+      <c r="L97" t="n">
         <v>33.33333333333333</v>
       </c>
     </row>
@@ -5118,9 +5704,15 @@
         </is>
       </c>
       <c r="I98" t="n">
+        <v>38</v>
+      </c>
+      <c r="J98" t="n">
         <v>69.09090909090909</v>
       </c>
-      <c r="J98" t="n">
+      <c r="K98" t="n">
+        <v>19</v>
+      </c>
+      <c r="L98" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -5166,9 +5758,15 @@
         </is>
       </c>
       <c r="I99" t="n">
+        <v>33</v>
+      </c>
+      <c r="J99" t="n">
         <v>60</v>
       </c>
-      <c r="J99" t="n">
+      <c r="K99" t="n">
+        <v>24</v>
+      </c>
+      <c r="L99" t="n">
         <v>80</v>
       </c>
     </row>
@@ -5214,9 +5812,15 @@
         </is>
       </c>
       <c r="I100" t="n">
+        <v>27</v>
+      </c>
+      <c r="J100" t="n">
         <v>49.09090909090909</v>
       </c>
-      <c r="J100" t="n">
+      <c r="K100" t="n">
+        <v>14</v>
+      </c>
+      <c r="L100" t="n">
         <v>46.66666666666666</v>
       </c>
     </row>
@@ -5262,9 +5866,15 @@
         </is>
       </c>
       <c r="I101" t="n">
+        <v>32</v>
+      </c>
+      <c r="J101" t="n">
         <v>58.18181818181818</v>
       </c>
-      <c r="J101" t="n">
+      <c r="K101" t="n">
+        <v>12</v>
+      </c>
+      <c r="L101" t="n">
         <v>40</v>
       </c>
     </row>
@@ -5310,9 +5920,15 @@
         </is>
       </c>
       <c r="I102" t="n">
+        <v>29</v>
+      </c>
+      <c r="J102" t="n">
         <v>52.72727272727272</v>
       </c>
-      <c r="J102" t="n">
+      <c r="K102" t="n">
+        <v>20</v>
+      </c>
+      <c r="L102" t="n">
         <v>66.66666666666666</v>
       </c>
     </row>
@@ -5358,9 +5974,15 @@
         </is>
       </c>
       <c r="I103" t="n">
+        <v>31</v>
+      </c>
+      <c r="J103" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J103" t="n">
+      <c r="K103" t="n">
+        <v>27</v>
+      </c>
+      <c r="L103" t="n">
         <v>90</v>
       </c>
     </row>
@@ -5406,9 +6028,15 @@
         </is>
       </c>
       <c r="I104" t="n">
+        <v>25</v>
+      </c>
+      <c r="J104" t="n">
         <v>45.45454545454545</v>
       </c>
-      <c r="J104" t="n">
+      <c r="K104" t="n">
+        <v>10</v>
+      </c>
+      <c r="L104" t="n">
         <v>33.33333333333333</v>
       </c>
     </row>
@@ -5454,9 +6082,15 @@
         </is>
       </c>
       <c r="I105" t="n">
+        <v>32</v>
+      </c>
+      <c r="J105" t="n">
         <v>58.18181818181818</v>
       </c>
-      <c r="J105" t="n">
+      <c r="K105" t="n">
+        <v>9</v>
+      </c>
+      <c r="L105" t="n">
         <v>30</v>
       </c>
     </row>
@@ -5502,9 +6136,15 @@
         </is>
       </c>
       <c r="I106" t="n">
+        <v>36</v>
+      </c>
+      <c r="J106" t="n">
         <v>65.45454545454545</v>
       </c>
-      <c r="J106" t="n">
+      <c r="K106" t="n">
+        <v>17</v>
+      </c>
+      <c r="L106" t="n">
         <v>56.66666666666666</v>
       </c>
     </row>
@@ -5550,9 +6190,15 @@
         </is>
       </c>
       <c r="I107" t="n">
+        <v>46</v>
+      </c>
+      <c r="J107" t="n">
         <v>83.63636363636363</v>
       </c>
-      <c r="J107" t="n">
+      <c r="K107" t="n">
+        <v>28</v>
+      </c>
+      <c r="L107" t="n">
         <v>93.33333333333333</v>
       </c>
     </row>
@@ -5598,9 +6244,15 @@
         </is>
       </c>
       <c r="I108" t="n">
+        <v>27</v>
+      </c>
+      <c r="J108" t="n">
         <v>49.09090909090909</v>
       </c>
-      <c r="J108" t="n">
+      <c r="K108" t="n">
+        <v>18</v>
+      </c>
+      <c r="L108" t="n">
         <v>60</v>
       </c>
     </row>
@@ -5646,9 +6298,15 @@
         </is>
       </c>
       <c r="I109" t="n">
+        <v>24</v>
+      </c>
+      <c r="J109" t="n">
         <v>43.63636363636363</v>
       </c>
-      <c r="J109" t="n">
+      <c r="K109" t="n">
+        <v>10</v>
+      </c>
+      <c r="L109" t="n">
         <v>33.33333333333333</v>
       </c>
     </row>
@@ -5694,9 +6352,15 @@
         </is>
       </c>
       <c r="I110" t="n">
+        <v>38</v>
+      </c>
+      <c r="J110" t="n">
         <v>69.09090909090909</v>
       </c>
-      <c r="J110" t="n">
+      <c r="K110" t="n">
+        <v>24</v>
+      </c>
+      <c r="L110" t="n">
         <v>80</v>
       </c>
     </row>
@@ -5742,9 +6406,15 @@
         </is>
       </c>
       <c r="I111" t="n">
+        <v>33</v>
+      </c>
+      <c r="J111" t="n">
         <v>60</v>
       </c>
-      <c r="J111" t="n">
+      <c r="K111" t="n">
+        <v>19</v>
+      </c>
+      <c r="L111" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -5790,9 +6460,15 @@
         </is>
       </c>
       <c r="I112" t="n">
+        <v>40</v>
+      </c>
+      <c r="J112" t="n">
         <v>72.72727272727273</v>
       </c>
-      <c r="J112" t="n">
+      <c r="K112" t="n">
+        <v>27</v>
+      </c>
+      <c r="L112" t="n">
         <v>90</v>
       </c>
     </row>
@@ -5838,9 +6514,15 @@
         </is>
       </c>
       <c r="I113" t="n">
+        <v>31</v>
+      </c>
+      <c r="J113" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J113" t="n">
+      <c r="K113" t="n">
+        <v>19</v>
+      </c>
+      <c r="L113" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -5886,9 +6568,15 @@
         </is>
       </c>
       <c r="I114" t="n">
+        <v>40</v>
+      </c>
+      <c r="J114" t="n">
         <v>72.72727272727273</v>
       </c>
-      <c r="J114" t="n">
+      <c r="K114" t="n">
+        <v>22</v>
+      </c>
+      <c r="L114" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -5934,9 +6622,15 @@
         </is>
       </c>
       <c r="I115" t="n">
+        <v>45</v>
+      </c>
+      <c r="J115" t="n">
         <v>81.81818181818183</v>
       </c>
-      <c r="J115" t="n">
+      <c r="K115" t="n">
+        <v>23</v>
+      </c>
+      <c r="L115" t="n">
         <v>76.66666666666667</v>
       </c>
     </row>
@@ -5982,9 +6676,15 @@
         </is>
       </c>
       <c r="I116" t="n">
+        <v>31</v>
+      </c>
+      <c r="J116" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J116" t="n">
+      <c r="K116" t="n">
+        <v>25</v>
+      </c>
+      <c r="L116" t="n">
         <v>83.33333333333334</v>
       </c>
     </row>
@@ -6030,9 +6730,15 @@
         </is>
       </c>
       <c r="I117" t="n">
+        <v>38</v>
+      </c>
+      <c r="J117" t="n">
         <v>69.09090909090909</v>
       </c>
-      <c r="J117" t="n">
+      <c r="K117" t="n">
+        <v>21</v>
+      </c>
+      <c r="L117" t="n">
         <v>70</v>
       </c>
     </row>
@@ -6078,9 +6784,15 @@
         </is>
       </c>
       <c r="I118" t="n">
+        <v>39</v>
+      </c>
+      <c r="J118" t="n">
         <v>70.90909090909091</v>
       </c>
-      <c r="J118" t="n">
+      <c r="K118" t="n">
+        <v>26</v>
+      </c>
+      <c r="L118" t="n">
         <v>86.66666666666667</v>
       </c>
     </row>
@@ -6126,9 +6838,15 @@
         </is>
       </c>
       <c r="I119" t="n">
+        <v>26</v>
+      </c>
+      <c r="J119" t="n">
         <v>47.27272727272727</v>
       </c>
-      <c r="J119" t="n">
+      <c r="K119" t="n">
+        <v>21</v>
+      </c>
+      <c r="L119" t="n">
         <v>70</v>
       </c>
     </row>
@@ -6174,9 +6892,15 @@
         </is>
       </c>
       <c r="I120" t="n">
+        <v>37</v>
+      </c>
+      <c r="J120" t="n">
         <v>67.27272727272727</v>
       </c>
-      <c r="J120" t="n">
+      <c r="K120" t="n">
+        <v>21</v>
+      </c>
+      <c r="L120" t="n">
         <v>70</v>
       </c>
     </row>
@@ -6222,9 +6946,15 @@
         </is>
       </c>
       <c r="I121" t="n">
+        <v>23</v>
+      </c>
+      <c r="J121" t="n">
         <v>41.81818181818181</v>
       </c>
-      <c r="J121" t="n">
+      <c r="K121" t="n">
+        <v>13</v>
+      </c>
+      <c r="L121" t="n">
         <v>43.33333333333334</v>
       </c>
     </row>
@@ -6270,9 +7000,15 @@
         </is>
       </c>
       <c r="I122" t="n">
+        <v>32</v>
+      </c>
+      <c r="J122" t="n">
         <v>58.18181818181818</v>
       </c>
-      <c r="J122" t="n">
+      <c r="K122" t="n">
+        <v>16</v>
+      </c>
+      <c r="L122" t="n">
         <v>53.33333333333334</v>
       </c>
     </row>
@@ -6318,9 +7054,15 @@
         </is>
       </c>
       <c r="I123" t="n">
+        <v>27</v>
+      </c>
+      <c r="J123" t="n">
         <v>49.09090909090909</v>
       </c>
-      <c r="J123" t="n">
+      <c r="K123" t="n">
+        <v>21</v>
+      </c>
+      <c r="L123" t="n">
         <v>70</v>
       </c>
     </row>
@@ -6366,9 +7108,15 @@
         </is>
       </c>
       <c r="I124" t="n">
+        <v>32</v>
+      </c>
+      <c r="J124" t="n">
         <v>58.18181818181818</v>
       </c>
-      <c r="J124" t="n">
+      <c r="K124" t="n">
+        <v>25</v>
+      </c>
+      <c r="L124" t="n">
         <v>83.33333333333334</v>
       </c>
     </row>
@@ -6414,9 +7162,15 @@
         </is>
       </c>
       <c r="I125" t="n">
+        <v>33</v>
+      </c>
+      <c r="J125" t="n">
         <v>60</v>
       </c>
-      <c r="J125" t="n">
+      <c r="K125" t="n">
+        <v>24</v>
+      </c>
+      <c r="L125" t="n">
         <v>80</v>
       </c>
     </row>
@@ -6462,9 +7216,15 @@
         </is>
       </c>
       <c r="I126" t="n">
+        <v>28</v>
+      </c>
+      <c r="J126" t="n">
         <v>50.90909090909091</v>
       </c>
-      <c r="J126" t="n">
+      <c r="K126" t="n">
+        <v>20</v>
+      </c>
+      <c r="L126" t="n">
         <v>66.66666666666666</v>
       </c>
     </row>
@@ -6510,9 +7270,15 @@
         </is>
       </c>
       <c r="I127" t="n">
+        <v>51</v>
+      </c>
+      <c r="J127" t="n">
         <v>92.72727272727272</v>
       </c>
-      <c r="J127" t="n">
+      <c r="K127" t="n">
+        <v>30</v>
+      </c>
+      <c r="L127" t="n">
         <v>100</v>
       </c>
     </row>
@@ -6558,9 +7324,15 @@
         </is>
       </c>
       <c r="I128" t="n">
+        <v>33</v>
+      </c>
+      <c r="J128" t="n">
         <v>60</v>
       </c>
-      <c r="J128" t="n">
+      <c r="K128" t="n">
+        <v>11</v>
+      </c>
+      <c r="L128" t="n">
         <v>36.66666666666666</v>
       </c>
     </row>
@@ -6606,9 +7378,15 @@
         </is>
       </c>
       <c r="I129" t="n">
+        <v>30</v>
+      </c>
+      <c r="J129" t="n">
         <v>54.54545454545454</v>
       </c>
-      <c r="J129" t="n">
+      <c r="K129" t="n">
+        <v>13</v>
+      </c>
+      <c r="L129" t="n">
         <v>43.33333333333334</v>
       </c>
     </row>
@@ -6654,9 +7432,15 @@
         </is>
       </c>
       <c r="I130" t="n">
+        <v>34</v>
+      </c>
+      <c r="J130" t="n">
         <v>61.81818181818181</v>
       </c>
-      <c r="J130" t="n">
+      <c r="K130" t="n">
+        <v>3</v>
+      </c>
+      <c r="L130" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6702,9 +7486,15 @@
         </is>
       </c>
       <c r="I131" t="n">
+        <v>45</v>
+      </c>
+      <c r="J131" t="n">
         <v>81.81818181818183</v>
       </c>
-      <c r="J131" t="n">
+      <c r="K131" t="n">
+        <v>15</v>
+      </c>
+      <c r="L131" t="n">
         <v>50</v>
       </c>
     </row>
@@ -6750,9 +7540,15 @@
         </is>
       </c>
       <c r="I132" t="n">
+        <v>21</v>
+      </c>
+      <c r="J132" t="n">
         <v>38.18181818181819</v>
       </c>
-      <c r="J132" t="n">
+      <c r="K132" t="n">
+        <v>8</v>
+      </c>
+      <c r="L132" t="n">
         <v>26.66666666666667</v>
       </c>
     </row>
@@ -6798,9 +7594,15 @@
         </is>
       </c>
       <c r="I133" t="n">
+        <v>40</v>
+      </c>
+      <c r="J133" t="n">
         <v>72.72727272727273</v>
       </c>
-      <c r="J133" t="n">
+      <c r="K133" t="n">
+        <v>15</v>
+      </c>
+      <c r="L133" t="n">
         <v>50</v>
       </c>
     </row>
@@ -6846,9 +7648,15 @@
         </is>
       </c>
       <c r="I134" t="n">
+        <v>51</v>
+      </c>
+      <c r="J134" t="n">
         <v>92.72727272727272</v>
       </c>
-      <c r="J134" t="n">
+      <c r="K134" t="n">
+        <v>25</v>
+      </c>
+      <c r="L134" t="n">
         <v>83.33333333333334</v>
       </c>
     </row>
@@ -6894,9 +7702,15 @@
         </is>
       </c>
       <c r="I135" t="n">
+        <v>28</v>
+      </c>
+      <c r="J135" t="n">
         <v>50.90909090909091</v>
       </c>
-      <c r="J135" t="n">
+      <c r="K135" t="n">
+        <v>19</v>
+      </c>
+      <c r="L135" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -6942,9 +7756,15 @@
         </is>
       </c>
       <c r="I136" t="n">
+        <v>34</v>
+      </c>
+      <c r="J136" t="n">
         <v>61.81818181818181</v>
       </c>
-      <c r="J136" t="n">
+      <c r="K136" t="n">
+        <v>21</v>
+      </c>
+      <c r="L136" t="n">
         <v>70</v>
       </c>
     </row>
@@ -6990,9 +7810,15 @@
         </is>
       </c>
       <c r="I137" t="n">
+        <v>31</v>
+      </c>
+      <c r="J137" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J137" t="n">
+      <c r="K137" t="n">
+        <v>19</v>
+      </c>
+      <c r="L137" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -7038,9 +7864,15 @@
         </is>
       </c>
       <c r="I138" t="n">
+        <v>28</v>
+      </c>
+      <c r="J138" t="n">
         <v>50.90909090909091</v>
       </c>
-      <c r="J138" t="n">
+      <c r="K138" t="n">
+        <v>10</v>
+      </c>
+      <c r="L138" t="n">
         <v>33.33333333333333</v>
       </c>
     </row>
@@ -7086,9 +7918,15 @@
         </is>
       </c>
       <c r="I139" t="n">
+        <v>28</v>
+      </c>
+      <c r="J139" t="n">
         <v>50.90909090909091</v>
       </c>
-      <c r="J139" t="n">
+      <c r="K139" t="n">
+        <v>17</v>
+      </c>
+      <c r="L139" t="n">
         <v>56.66666666666666</v>
       </c>
     </row>
@@ -7134,9 +7972,15 @@
         </is>
       </c>
       <c r="I140" t="n">
+        <v>39</v>
+      </c>
+      <c r="J140" t="n">
         <v>70.90909090909091</v>
       </c>
-      <c r="J140" t="n">
+      <c r="K140" t="n">
+        <v>8</v>
+      </c>
+      <c r="L140" t="n">
         <v>26.66666666666667</v>
       </c>
     </row>
@@ -7182,9 +8026,15 @@
         </is>
       </c>
       <c r="I141" t="n">
+        <v>35</v>
+      </c>
+      <c r="J141" t="n">
         <v>63.63636363636363</v>
       </c>
-      <c r="J141" t="n">
+      <c r="K141" t="n">
+        <v>22</v>
+      </c>
+      <c r="L141" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -7230,9 +8080,15 @@
         </is>
       </c>
       <c r="I142" t="n">
+        <v>30</v>
+      </c>
+      <c r="J142" t="n">
         <v>54.54545454545454</v>
       </c>
-      <c r="J142" t="n">
+      <c r="K142" t="n">
+        <v>18</v>
+      </c>
+      <c r="L142" t="n">
         <v>60</v>
       </c>
     </row>
@@ -7278,9 +8134,15 @@
         </is>
       </c>
       <c r="I143" t="n">
+        <v>36</v>
+      </c>
+      <c r="J143" t="n">
         <v>65.45454545454545</v>
       </c>
-      <c r="J143" t="n">
+      <c r="K143" t="n">
+        <v>22</v>
+      </c>
+      <c r="L143" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -7326,9 +8188,15 @@
         </is>
       </c>
       <c r="I144" t="n">
+        <v>28</v>
+      </c>
+      <c r="J144" t="n">
         <v>50.90909090909091</v>
       </c>
-      <c r="J144" t="n">
+      <c r="K144" t="n">
+        <v>21</v>
+      </c>
+      <c r="L144" t="n">
         <v>70</v>
       </c>
     </row>
@@ -7374,9 +8242,15 @@
         </is>
       </c>
       <c r="I145" t="n">
+        <v>32</v>
+      </c>
+      <c r="J145" t="n">
         <v>58.18181818181818</v>
       </c>
-      <c r="J145" t="n">
+      <c r="K145" t="n">
+        <v>16</v>
+      </c>
+      <c r="L145" t="n">
         <v>53.33333333333334</v>
       </c>
     </row>
@@ -7422,9 +8296,15 @@
         </is>
       </c>
       <c r="I146" t="n">
+        <v>31</v>
+      </c>
+      <c r="J146" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J146" t="n">
+      <c r="K146" t="n">
+        <v>11</v>
+      </c>
+      <c r="L146" t="n">
         <v>36.66666666666666</v>
       </c>
     </row>
@@ -7470,9 +8350,15 @@
         </is>
       </c>
       <c r="I147" t="n">
+        <v>44</v>
+      </c>
+      <c r="J147" t="n">
         <v>80</v>
       </c>
-      <c r="J147" t="n">
+      <c r="K147" t="n">
+        <v>21</v>
+      </c>
+      <c r="L147" t="n">
         <v>70</v>
       </c>
     </row>
@@ -7518,9 +8404,15 @@
         </is>
       </c>
       <c r="I148" t="n">
+        <v>28</v>
+      </c>
+      <c r="J148" t="n">
         <v>50.90909090909091</v>
       </c>
-      <c r="J148" t="n">
+      <c r="K148" t="n">
+        <v>11</v>
+      </c>
+      <c r="L148" t="n">
         <v>36.66666666666666</v>
       </c>
     </row>
@@ -7566,9 +8458,15 @@
         </is>
       </c>
       <c r="I149" t="n">
+        <v>31</v>
+      </c>
+      <c r="J149" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J149" t="n">
+      <c r="K149" t="n">
+        <v>6</v>
+      </c>
+      <c r="L149" t="n">
         <v>20</v>
       </c>
     </row>
@@ -7614,9 +8512,15 @@
         </is>
       </c>
       <c r="I150" t="n">
+        <v>27</v>
+      </c>
+      <c r="J150" t="n">
         <v>49.09090909090909</v>
       </c>
-      <c r="J150" t="n">
+      <c r="K150" t="n">
+        <v>9</v>
+      </c>
+      <c r="L150" t="n">
         <v>30</v>
       </c>
     </row>
@@ -7662,9 +8566,15 @@
         </is>
       </c>
       <c r="I151" t="n">
+        <v>30</v>
+      </c>
+      <c r="J151" t="n">
         <v>54.54545454545454</v>
       </c>
-      <c r="J151" t="n">
+      <c r="K151" t="n">
+        <v>27</v>
+      </c>
+      <c r="L151" t="n">
         <v>90</v>
       </c>
     </row>
@@ -7710,9 +8620,15 @@
         </is>
       </c>
       <c r="I152" t="n">
+        <v>51</v>
+      </c>
+      <c r="J152" t="n">
         <v>92.72727272727272</v>
       </c>
-      <c r="J152" t="n">
+      <c r="K152" t="n">
+        <v>28</v>
+      </c>
+      <c r="L152" t="n">
         <v>93.33333333333333</v>
       </c>
     </row>
@@ -7758,9 +8674,15 @@
         </is>
       </c>
       <c r="I153" t="n">
+        <v>48</v>
+      </c>
+      <c r="J153" t="n">
         <v>87.27272727272727</v>
       </c>
-      <c r="J153" t="n">
+      <c r="K153" t="n">
+        <v>13</v>
+      </c>
+      <c r="L153" t="n">
         <v>43.33333333333334</v>
       </c>
     </row>
@@ -7806,9 +8728,15 @@
         </is>
       </c>
       <c r="I154" t="n">
+        <v>29</v>
+      </c>
+      <c r="J154" t="n">
         <v>52.72727272727272</v>
       </c>
-      <c r="J154" t="n">
+      <c r="K154" t="n">
+        <v>20</v>
+      </c>
+      <c r="L154" t="n">
         <v>66.66666666666666</v>
       </c>
     </row>
@@ -7854,9 +8782,15 @@
         </is>
       </c>
       <c r="I155" t="n">
+        <v>33</v>
+      </c>
+      <c r="J155" t="n">
         <v>60</v>
       </c>
-      <c r="J155" t="n">
+      <c r="K155" t="n">
+        <v>4</v>
+      </c>
+      <c r="L155" t="n">
         <v>13.33333333333333</v>
       </c>
     </row>
@@ -7902,9 +8836,15 @@
         </is>
       </c>
       <c r="I156" t="n">
+        <v>21</v>
+      </c>
+      <c r="J156" t="n">
         <v>38.18181818181819</v>
       </c>
-      <c r="J156" t="n">
+      <c r="K156" t="n">
+        <v>20</v>
+      </c>
+      <c r="L156" t="n">
         <v>66.66666666666666</v>
       </c>
     </row>
@@ -7950,9 +8890,15 @@
         </is>
       </c>
       <c r="I157" t="n">
+        <v>38</v>
+      </c>
+      <c r="J157" t="n">
         <v>69.09090909090909</v>
       </c>
-      <c r="J157" t="n">
+      <c r="K157" t="n">
+        <v>24</v>
+      </c>
+      <c r="L157" t="n">
         <v>80</v>
       </c>
     </row>
@@ -7998,9 +8944,15 @@
         </is>
       </c>
       <c r="I158" t="n">
+        <v>33</v>
+      </c>
+      <c r="J158" t="n">
         <v>60</v>
       </c>
-      <c r="J158" t="n">
+      <c r="K158" t="n">
+        <v>23</v>
+      </c>
+      <c r="L158" t="n">
         <v>76.66666666666667</v>
       </c>
     </row>
@@ -8046,9 +8998,15 @@
         </is>
       </c>
       <c r="I159" t="n">
+        <v>23</v>
+      </c>
+      <c r="J159" t="n">
         <v>41.81818181818181</v>
       </c>
-      <c r="J159" t="n">
+      <c r="K159" t="n">
+        <v>13</v>
+      </c>
+      <c r="L159" t="n">
         <v>43.33333333333334</v>
       </c>
     </row>
@@ -8094,9 +9052,15 @@
         </is>
       </c>
       <c r="I160" t="n">
+        <v>31</v>
+      </c>
+      <c r="J160" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J160" t="n">
+      <c r="K160" t="n">
+        <v>18</v>
+      </c>
+      <c r="L160" t="n">
         <v>60</v>
       </c>
     </row>
@@ -8142,9 +9106,15 @@
         </is>
       </c>
       <c r="I161" t="n">
+        <v>26</v>
+      </c>
+      <c r="J161" t="n">
         <v>47.27272727272727</v>
       </c>
-      <c r="J161" t="n">
+      <c r="K161" t="n">
+        <v>16</v>
+      </c>
+      <c r="L161" t="n">
         <v>53.33333333333334</v>
       </c>
     </row>
@@ -8190,9 +9160,15 @@
         </is>
       </c>
       <c r="I162" t="n">
+        <v>32</v>
+      </c>
+      <c r="J162" t="n">
         <v>58.18181818181818</v>
       </c>
-      <c r="J162" t="n">
+      <c r="K162" t="n">
+        <v>26</v>
+      </c>
+      <c r="L162" t="n">
         <v>86.66666666666667</v>
       </c>
     </row>
@@ -8238,9 +9214,15 @@
         </is>
       </c>
       <c r="I163" t="n">
+        <v>42</v>
+      </c>
+      <c r="J163" t="n">
         <v>76.36363636363637</v>
       </c>
-      <c r="J163" t="n">
+      <c r="K163" t="n">
+        <v>20</v>
+      </c>
+      <c r="L163" t="n">
         <v>66.66666666666666</v>
       </c>
     </row>
@@ -8286,9 +9268,15 @@
         </is>
       </c>
       <c r="I164" t="n">
+        <v>35</v>
+      </c>
+      <c r="J164" t="n">
         <v>63.63636363636363</v>
       </c>
-      <c r="J164" t="n">
+      <c r="K164" t="n">
+        <v>21</v>
+      </c>
+      <c r="L164" t="n">
         <v>70</v>
       </c>
     </row>
@@ -8334,9 +9322,15 @@
         </is>
       </c>
       <c r="I165" t="n">
+        <v>41</v>
+      </c>
+      <c r="J165" t="n">
         <v>74.54545454545455</v>
       </c>
-      <c r="J165" t="n">
+      <c r="K165" t="n">
+        <v>19</v>
+      </c>
+      <c r="L165" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -8382,9 +9376,15 @@
         </is>
       </c>
       <c r="I166" t="n">
+        <v>43</v>
+      </c>
+      <c r="J166" t="n">
         <v>78.18181818181819</v>
       </c>
-      <c r="J166" t="n">
+      <c r="K166" t="n">
+        <v>25</v>
+      </c>
+      <c r="L166" t="n">
         <v>83.33333333333334</v>
       </c>
     </row>
@@ -8430,9 +9430,15 @@
         </is>
       </c>
       <c r="I167" t="n">
+        <v>38</v>
+      </c>
+      <c r="J167" t="n">
         <v>69.09090909090909</v>
       </c>
-      <c r="J167" t="n">
+      <c r="K167" t="n">
+        <v>22</v>
+      </c>
+      <c r="L167" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -8478,9 +9484,15 @@
         </is>
       </c>
       <c r="I168" t="n">
+        <v>31</v>
+      </c>
+      <c r="J168" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J168" t="n">
+      <c r="K168" t="n">
+        <v>21</v>
+      </c>
+      <c r="L168" t="n">
         <v>70</v>
       </c>
     </row>
@@ -8526,9 +9538,15 @@
         </is>
       </c>
       <c r="I169" t="n">
+        <v>34</v>
+      </c>
+      <c r="J169" t="n">
         <v>61.81818181818181</v>
       </c>
-      <c r="J169" t="n">
+      <c r="K169" t="n">
+        <v>25</v>
+      </c>
+      <c r="L169" t="n">
         <v>83.33333333333334</v>
       </c>
     </row>
@@ -8574,9 +9592,15 @@
         </is>
       </c>
       <c r="I170" t="n">
+        <v>35</v>
+      </c>
+      <c r="J170" t="n">
         <v>63.63636363636363</v>
       </c>
-      <c r="J170" t="n">
+      <c r="K170" t="n">
+        <v>21</v>
+      </c>
+      <c r="L170" t="n">
         <v>70</v>
       </c>
     </row>
@@ -8622,9 +9646,15 @@
         </is>
       </c>
       <c r="I171" t="n">
+        <v>17</v>
+      </c>
+      <c r="J171" t="n">
         <v>30.90909090909091</v>
       </c>
-      <c r="J171" t="n">
+      <c r="K171" t="n">
+        <v>10</v>
+      </c>
+      <c r="L171" t="n">
         <v>33.33333333333333</v>
       </c>
     </row>
@@ -8670,9 +9700,15 @@
         </is>
       </c>
       <c r="I172" t="n">
+        <v>29</v>
+      </c>
+      <c r="J172" t="n">
         <v>52.72727272727272</v>
       </c>
-      <c r="J172" t="n">
+      <c r="K172" t="n">
+        <v>22</v>
+      </c>
+      <c r="L172" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -8718,9 +9754,15 @@
         </is>
       </c>
       <c r="I173" t="n">
+        <v>29</v>
+      </c>
+      <c r="J173" t="n">
         <v>52.72727272727272</v>
       </c>
-      <c r="J173" t="n">
+      <c r="K173" t="n">
+        <v>19</v>
+      </c>
+      <c r="L173" t="n">
         <v>63.33333333333333</v>
       </c>
     </row>
@@ -8766,9 +9808,15 @@
         </is>
       </c>
       <c r="I174" t="n">
+        <v>37</v>
+      </c>
+      <c r="J174" t="n">
         <v>67.27272727272727</v>
       </c>
-      <c r="J174" t="n">
+      <c r="K174" t="n">
+        <v>20</v>
+      </c>
+      <c r="L174" t="n">
         <v>66.66666666666666</v>
       </c>
     </row>
@@ -8814,9 +9862,15 @@
         </is>
       </c>
       <c r="I175" t="n">
+        <v>30</v>
+      </c>
+      <c r="J175" t="n">
         <v>54.54545454545454</v>
       </c>
-      <c r="J175" t="n">
+      <c r="K175" t="n">
+        <v>10</v>
+      </c>
+      <c r="L175" t="n">
         <v>33.33333333333333</v>
       </c>
     </row>
@@ -8862,9 +9916,15 @@
         </is>
       </c>
       <c r="I176" t="n">
+        <v>49</v>
+      </c>
+      <c r="J176" t="n">
         <v>89.09090909090909</v>
       </c>
-      <c r="J176" t="n">
+      <c r="K176" t="n">
+        <v>28</v>
+      </c>
+      <c r="L176" t="n">
         <v>93.33333333333333</v>
       </c>
     </row>
@@ -8910,9 +9970,15 @@
         </is>
       </c>
       <c r="I177" t="n">
+        <v>35</v>
+      </c>
+      <c r="J177" t="n">
         <v>63.63636363636363</v>
       </c>
-      <c r="J177" t="n">
+      <c r="K177" t="n">
+        <v>25</v>
+      </c>
+      <c r="L177" t="n">
         <v>83.33333333333334</v>
       </c>
     </row>
@@ -8958,9 +10024,15 @@
         </is>
       </c>
       <c r="I178" t="n">
+        <v>25</v>
+      </c>
+      <c r="J178" t="n">
         <v>45.45454545454545</v>
       </c>
-      <c r="J178" t="n">
+      <c r="K178" t="n">
+        <v>16</v>
+      </c>
+      <c r="L178" t="n">
         <v>53.33333333333334</v>
       </c>
     </row>
@@ -9006,9 +10078,15 @@
         </is>
       </c>
       <c r="I179" t="n">
+        <v>29</v>
+      </c>
+      <c r="J179" t="n">
         <v>52.72727272727272</v>
       </c>
-      <c r="J179" t="n">
+      <c r="K179" t="n">
+        <v>18</v>
+      </c>
+      <c r="L179" t="n">
         <v>60</v>
       </c>
     </row>
@@ -9054,9 +10132,15 @@
         </is>
       </c>
       <c r="I180" t="n">
+        <v>40</v>
+      </c>
+      <c r="J180" t="n">
         <v>72.72727272727273</v>
       </c>
-      <c r="J180" t="n">
+      <c r="K180" t="n">
+        <v>15</v>
+      </c>
+      <c r="L180" t="n">
         <v>50</v>
       </c>
     </row>
@@ -9102,9 +10186,15 @@
         </is>
       </c>
       <c r="I181" t="n">
+        <v>38</v>
+      </c>
+      <c r="J181" t="n">
         <v>69.09090909090909</v>
       </c>
-      <c r="J181" t="n">
+      <c r="K181" t="n">
+        <v>18</v>
+      </c>
+      <c r="L181" t="n">
         <v>60</v>
       </c>
     </row>
@@ -9150,9 +10240,15 @@
         </is>
       </c>
       <c r="I182" t="n">
+        <v>29</v>
+      </c>
+      <c r="J182" t="n">
         <v>52.72727272727272</v>
       </c>
-      <c r="J182" t="n">
+      <c r="K182" t="n">
+        <v>18</v>
+      </c>
+      <c r="L182" t="n">
         <v>60</v>
       </c>
     </row>
@@ -9198,9 +10294,15 @@
         </is>
       </c>
       <c r="I183" t="n">
+        <v>34</v>
+      </c>
+      <c r="J183" t="n">
         <v>61.81818181818181</v>
       </c>
-      <c r="J183" t="n">
+      <c r="K183" t="n">
+        <v>23</v>
+      </c>
+      <c r="L183" t="n">
         <v>76.66666666666667</v>
       </c>
     </row>
@@ -9246,9 +10348,15 @@
         </is>
       </c>
       <c r="I184" t="n">
+        <v>45</v>
+      </c>
+      <c r="J184" t="n">
         <v>81.81818181818183</v>
       </c>
-      <c r="J184" t="n">
+      <c r="K184" t="n">
+        <v>23</v>
+      </c>
+      <c r="L184" t="n">
         <v>76.66666666666667</v>
       </c>
     </row>
@@ -9294,9 +10402,15 @@
         </is>
       </c>
       <c r="I185" t="n">
+        <v>40</v>
+      </c>
+      <c r="J185" t="n">
         <v>72.72727272727273</v>
       </c>
-      <c r="J185" t="n">
+      <c r="K185" t="n">
+        <v>14</v>
+      </c>
+      <c r="L185" t="n">
         <v>46.66666666666666</v>
       </c>
     </row>
@@ -9342,9 +10456,15 @@
         </is>
       </c>
       <c r="I186" t="n">
+        <v>37</v>
+      </c>
+      <c r="J186" t="n">
         <v>67.27272727272727</v>
       </c>
-      <c r="J186" t="n">
+      <c r="K186" t="n">
+        <v>22</v>
+      </c>
+      <c r="L186" t="n">
         <v>73.33333333333333</v>
       </c>
     </row>
@@ -9390,9 +10510,15 @@
         </is>
       </c>
       <c r="I187" t="n">
+        <v>31</v>
+      </c>
+      <c r="J187" t="n">
         <v>56.36363636363636</v>
       </c>
-      <c r="J187" t="n">
+      <c r="K187" t="n">
+        <v>14</v>
+      </c>
+      <c r="L187" t="n">
         <v>46.66666666666666</v>
       </c>
     </row>
@@ -9438,9 +10564,15 @@
         </is>
       </c>
       <c r="I188" t="n">
+        <v>45</v>
+      </c>
+      <c r="J188" t="n">
         <v>81.81818181818183</v>
       </c>
-      <c r="J188" t="n">
+      <c r="K188" t="n">
+        <v>28</v>
+      </c>
+      <c r="L188" t="n">
         <v>93.33333333333333</v>
       </c>
     </row>

</xml_diff>